<commit_message>
final results for greedy
</commit_message>
<xml_diff>
--- a/results/cluster_ga/UAVs10_GRID13/revenue/UAVs10_GRID13_cluster_ga.xlsx
+++ b/results/cluster_ga/UAVs10_GRID13/revenue/UAVs10_GRID13_cluster_ga.xlsx
@@ -582,37 +582,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6983626669971272</v>
+        <v>142.8097187500098</v>
       </c>
       <c r="C2" t="n">
-        <v>30.64089997739027</v>
+        <v>45.14188163425587</v>
       </c>
       <c r="D2" t="n">
         <v>54.95758115613536</v>
       </c>
       <c r="E2" t="n">
-        <v>33.31822946519443</v>
+        <v>36.19903883038042</v>
       </c>
       <c r="F2" t="n">
-        <v>37.33193623655075</v>
+        <v>41.75699241485186</v>
       </c>
       <c r="G2" t="n">
-        <v>50.39455743627249</v>
+        <v>50.21654431734949</v>
       </c>
       <c r="H2" t="n">
-        <v>51.04610831284837</v>
+        <v>50.97632154671587</v>
       </c>
       <c r="I2" t="n">
-        <v>44.74626962227806</v>
+        <v>48.16638727751</v>
       </c>
       <c r="J2" t="n">
-        <v>37.6157323181909</v>
+        <v>38.48408297556348</v>
       </c>
       <c r="K2" t="n">
-        <v>31.18537199024974</v>
+        <v>43.73221447941854</v>
       </c>
       <c r="L2" t="n">
-        <v>44.87351461691586</v>
+        <v>55.51312198388092</v>
       </c>
     </row>
   </sheetData>
@@ -696,34 +696,34 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6596656669862568</v>
+        <v>128.1824172920315</v>
       </c>
       <c r="C2" t="n">
-        <v>57.87190614286904</v>
+        <v>57.43923003300519</v>
       </c>
       <c r="D2" t="n">
-        <v>50.1567681642511</v>
+        <v>50.62647609823353</v>
       </c>
       <c r="E2" t="n">
-        <v>37.95624928963225</v>
+        <v>40.28081065527178</v>
       </c>
       <c r="F2" t="n">
-        <v>39.3368374898076</v>
+        <v>45.2437971283142</v>
       </c>
       <c r="G2" t="n">
-        <v>51.35001834500388</v>
+        <v>50.76272566579165</v>
       </c>
       <c r="H2" t="n">
-        <v>48.01864917027741</v>
+        <v>49.0112439874372</v>
       </c>
       <c r="I2" t="n">
         <v>28.98641850957833</v>
       </c>
       <c r="J2" t="n">
-        <v>45.80978215696096</v>
+        <v>45.84859657759117</v>
       </c>
       <c r="K2" t="n">
-        <v>34.09415816432296</v>
+        <v>34.62864858356834</v>
       </c>
       <c r="L2" t="n">
         <v>39.69527329371493</v>
@@ -810,34 +810,34 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6619732920080423</v>
+        <v>135.898960874998</v>
       </c>
       <c r="C2" t="n">
-        <v>36.08463815328094</v>
+        <v>37.96030347045147</v>
       </c>
       <c r="D2" t="n">
-        <v>56.11171233196637</v>
+        <v>56.11360271637923</v>
       </c>
       <c r="E2" t="n">
-        <v>33.47967049535403</v>
+        <v>36.1637248643159</v>
       </c>
       <c r="F2" t="n">
-        <v>50.9834111485218</v>
+        <v>55.09363522738357</v>
       </c>
       <c r="G2" t="n">
-        <v>34.01159807375255</v>
+        <v>33.61220094730393</v>
       </c>
       <c r="H2" t="n">
-        <v>43.41395956391906</v>
+        <v>49.4601162968608</v>
       </c>
       <c r="I2" t="n">
-        <v>39.13578350381007</v>
+        <v>49.16143923503974</v>
       </c>
       <c r="J2" t="n">
-        <v>37.47512181949529</v>
+        <v>41.26421103317281</v>
       </c>
       <c r="K2" t="n">
-        <v>45.61215807000271</v>
+        <v>51.49232708894244</v>
       </c>
       <c r="L2" t="n">
         <v>49.65267055078131</v>
@@ -924,37 +924,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7063138749799691</v>
+        <v>138.5075207499904</v>
       </c>
       <c r="C2" t="n">
-        <v>32.13045921266482</v>
+        <v>33.93176329011389</v>
       </c>
       <c r="D2" t="n">
-        <v>37.0455615997689</v>
+        <v>40.22783050409188</v>
       </c>
       <c r="E2" t="n">
-        <v>43.70445636387205</v>
+        <v>48.03200431492663</v>
       </c>
       <c r="F2" t="n">
-        <v>43.74280464795716</v>
+        <v>45.75903558481762</v>
       </c>
       <c r="G2" t="n">
-        <v>46.82165824909097</v>
+        <v>49.60663757525329</v>
       </c>
       <c r="H2" t="n">
-        <v>37.53198776943967</v>
+        <v>43.93377595387843</v>
       </c>
       <c r="I2" t="n">
-        <v>53.94583092444118</v>
+        <v>54.94327554063093</v>
       </c>
       <c r="J2" t="n">
-        <v>43.87067001562225</v>
+        <v>43.15213967483799</v>
       </c>
       <c r="K2" t="n">
-        <v>45.14753902842818</v>
+        <v>40.65004634046728</v>
       </c>
       <c r="L2" t="n">
-        <v>34.86817228467043</v>
+        <v>35.33542881518159</v>
       </c>
     </row>
   </sheetData>
@@ -1038,37 +1038,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6980081250076182</v>
+        <v>135.7721852920367</v>
       </c>
       <c r="C2" t="n">
-        <v>44.47585251250133</v>
+        <v>45.42790730964956</v>
       </c>
       <c r="D2" t="n">
         <v>23.80614835033256</v>
       </c>
       <c r="E2" t="n">
-        <v>42.41847193263498</v>
+        <v>42.72068231205601</v>
       </c>
       <c r="F2" t="n">
-        <v>26.04260906620736</v>
+        <v>26.20756978565871</v>
       </c>
       <c r="G2" t="n">
-        <v>42.01046708697654</v>
+        <v>44.40498953007175</v>
       </c>
       <c r="H2" t="n">
-        <v>42.571843191264</v>
+        <v>44.18086545338758</v>
       </c>
       <c r="I2" t="n">
-        <v>46.27663492117146</v>
+        <v>51.55808721689127</v>
       </c>
       <c r="J2" t="n">
-        <v>49.82552063914846</v>
+        <v>50.25161806462476</v>
       </c>
       <c r="K2" t="n">
-        <v>46.27755926558002</v>
+        <v>49.26001704034461</v>
       </c>
       <c r="L2" t="n">
-        <v>45.00168792151792</v>
+        <v>54.47820164366347</v>
       </c>
     </row>
   </sheetData>
@@ -1152,37 +1152,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6688979580067098</v>
+        <v>131.0425190830138</v>
       </c>
       <c r="C2" t="n">
         <v>39.65626125068405</v>
       </c>
       <c r="D2" t="n">
-        <v>45.63074196540773</v>
+        <v>45.73208297532683</v>
       </c>
       <c r="E2" t="n">
-        <v>43.77639450019177</v>
+        <v>43.87226755484874</v>
       </c>
       <c r="F2" t="n">
-        <v>41.10399825861794</v>
+        <v>41.49664342320297</v>
       </c>
       <c r="G2" t="n">
-        <v>31.62400369112984</v>
+        <v>33.01763719961872</v>
       </c>
       <c r="H2" t="n">
-        <v>55.35709667514531</v>
+        <v>56.07461799572249</v>
       </c>
       <c r="I2" t="n">
-        <v>45.86901161235007</v>
+        <v>45.91284244162996</v>
       </c>
       <c r="J2" t="n">
-        <v>44.84659554142877</v>
+        <v>59.59795525092345</v>
       </c>
       <c r="K2" t="n">
         <v>51.1032547168081</v>
       </c>
       <c r="L2" t="n">
-        <v>37.25034136975769</v>
+        <v>42.85028129238444</v>
       </c>
     </row>
   </sheetData>
@@ -1266,37 +1266,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7385846669785678</v>
+        <v>146.5444977079751</v>
       </c>
       <c r="C2" t="n">
-        <v>47.44387711238274</v>
+        <v>49.69580792716552</v>
       </c>
       <c r="D2" t="n">
-        <v>37.42045151489278</v>
+        <v>56.16184420217485</v>
       </c>
       <c r="E2" t="n">
-        <v>48.81310585120038</v>
+        <v>58.23066180121293</v>
       </c>
       <c r="F2" t="n">
-        <v>48.88768401390119</v>
+        <v>50.98900653386969</v>
       </c>
       <c r="G2" t="n">
-        <v>33.05082770783759</v>
+        <v>33.41063675226246</v>
       </c>
       <c r="H2" t="n">
-        <v>33.79654494940704</v>
+        <v>36.3702443848461</v>
       </c>
       <c r="I2" t="n">
-        <v>59.89149086237198</v>
+        <v>51.74080429352695</v>
       </c>
       <c r="J2" t="n">
-        <v>45.75709499193413</v>
+        <v>56.16139346062413</v>
       </c>
       <c r="K2" t="n">
-        <v>31.01826134950525</v>
+        <v>36.39721956368361</v>
       </c>
       <c r="L2" t="n">
-        <v>40.04045266639684</v>
+        <v>48.05084643662077</v>
       </c>
     </row>
   </sheetData>
@@ -1380,37 +1380,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.721073874970898</v>
+        <v>143.1646321250009</v>
       </c>
       <c r="C2" t="n">
-        <v>34.8363072611165</v>
+        <v>38.8720015922416</v>
       </c>
       <c r="D2" t="n">
-        <v>34.24873817084637</v>
+        <v>36.20369829759571</v>
       </c>
       <c r="E2" t="n">
-        <v>36.42951757366099</v>
+        <v>42.04029132282823</v>
       </c>
       <c r="F2" t="n">
-        <v>34.99435313740901</v>
+        <v>37.9752167278171</v>
       </c>
       <c r="G2" t="n">
-        <v>60.94285038105556</v>
+        <v>61.31719453655993</v>
       </c>
       <c r="H2" t="n">
-        <v>42.24047619155725</v>
+        <v>48.87361582921463</v>
       </c>
       <c r="I2" t="n">
-        <v>42.48202703541318</v>
+        <v>42.92441970794182</v>
       </c>
       <c r="J2" t="n">
-        <v>34.05280075874438</v>
+        <v>35.49354348760635</v>
       </c>
       <c r="K2" t="n">
-        <v>43.28071244242095</v>
+        <v>48.03745506173735</v>
       </c>
       <c r="L2" t="n">
-        <v>39.952329147895</v>
+        <v>40.02441174666329</v>
       </c>
     </row>
   </sheetData>
@@ -1494,37 +1494,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7023369579692371</v>
+        <v>141.1735491250292</v>
       </c>
       <c r="C2" t="n">
-        <v>38.73913112929698</v>
+        <v>39.01459154546444</v>
       </c>
       <c r="D2" t="n">
-        <v>49.71094319306505</v>
+        <v>49.33008350669586</v>
       </c>
       <c r="E2" t="n">
         <v>26.19629428815284</v>
       </c>
       <c r="F2" t="n">
-        <v>29.15870468671938</v>
+        <v>32.11469791338786</v>
       </c>
       <c r="G2" t="n">
-        <v>45.64948359006539</v>
+        <v>45.64948359006538</v>
       </c>
       <c r="H2" t="n">
-        <v>39.21935982132701</v>
+        <v>49.61333437497171</v>
       </c>
       <c r="I2" t="n">
-        <v>40.04035580857041</v>
+        <v>46.11797182359032</v>
       </c>
       <c r="J2" t="n">
-        <v>35.09419345362161</v>
+        <v>47.15117938033017</v>
       </c>
       <c r="K2" t="n">
-        <v>38.55930480367332</v>
+        <v>41.47566101657837</v>
       </c>
       <c r="L2" t="n">
-        <v>50.6070712401276</v>
+        <v>50.71132417422174</v>
       </c>
     </row>
   </sheetData>
@@ -1608,37 +1608,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7582349170115776</v>
+        <v>144.1620770420413</v>
       </c>
       <c r="C2" t="n">
-        <v>50.90099963471025</v>
+        <v>51.1056359373409</v>
       </c>
       <c r="D2" t="n">
-        <v>49.23685387701571</v>
+        <v>58.3186833443712</v>
       </c>
       <c r="E2" t="n">
-        <v>31.63861033326786</v>
+        <v>32.42096252435717</v>
       </c>
       <c r="F2" t="n">
-        <v>30.09996616774669</v>
+        <v>30.35953790246194</v>
       </c>
       <c r="G2" t="n">
-        <v>32.81686397124536</v>
+        <v>34.0467211584094</v>
       </c>
       <c r="H2" t="n">
-        <v>49.19874994158165</v>
+        <v>49.50056018622008</v>
       </c>
       <c r="I2" t="n">
-        <v>39.90305385863496</v>
+        <v>44.53306637377634</v>
       </c>
       <c r="J2" t="n">
-        <v>38.88872601302403</v>
+        <v>48.0441294651579</v>
       </c>
       <c r="K2" t="n">
-        <v>35.35101256418555</v>
+        <v>42.703005153964</v>
       </c>
       <c r="L2" t="n">
-        <v>34.57086230284349</v>
+        <v>41.3855059558805</v>
       </c>
     </row>
   </sheetData>
@@ -1722,37 +1722,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7590186249581166</v>
+        <v>132.5768951670034</v>
       </c>
       <c r="C2" t="n">
-        <v>49.54504955455143</v>
+        <v>49.57537689905789</v>
       </c>
       <c r="D2" t="n">
-        <v>24.57915195103729</v>
+        <v>24.63863411157709</v>
       </c>
       <c r="E2" t="n">
-        <v>41.34962180414737</v>
+        <v>44.33248895858877</v>
       </c>
       <c r="F2" t="n">
-        <v>44.52713028637036</v>
+        <v>50.26882015757416</v>
       </c>
       <c r="G2" t="n">
-        <v>21.11278503982513</v>
+        <v>21.23356882806142</v>
       </c>
       <c r="H2" t="n">
-        <v>59.63987095091296</v>
+        <v>60.12558212973764</v>
       </c>
       <c r="I2" t="n">
-        <v>54.751932755734</v>
+        <v>53.87519883384122</v>
       </c>
       <c r="J2" t="n">
-        <v>33.58237371284634</v>
+        <v>37.92692139706904</v>
       </c>
       <c r="K2" t="n">
-        <v>45.90080416861716</v>
+        <v>46.34185328225757</v>
       </c>
       <c r="L2" t="n">
-        <v>35.65562138654372</v>
+        <v>36.1151502448029</v>
       </c>
     </row>
   </sheetData>
@@ -1836,37 +1836,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6820087080122903</v>
+        <v>135.5944071250269</v>
       </c>
       <c r="C2" t="n">
-        <v>44.62087358635117</v>
+        <v>47.53849362633034</v>
       </c>
       <c r="D2" t="n">
-        <v>39.93752244469111</v>
+        <v>44.25464541904751</v>
       </c>
       <c r="E2" t="n">
-        <v>36.188599513144</v>
+        <v>44.92196297467593</v>
       </c>
       <c r="F2" t="n">
-        <v>40.16787518717445</v>
+        <v>44.56883192843088</v>
       </c>
       <c r="G2" t="n">
-        <v>49.01708606989771</v>
+        <v>48.19834586966078</v>
       </c>
       <c r="H2" t="n">
-        <v>43.49996334708031</v>
+        <v>47.33832734020494</v>
       </c>
       <c r="I2" t="n">
-        <v>45.9942508325083</v>
+        <v>46.26183861207563</v>
       </c>
       <c r="J2" t="n">
-        <v>35.23845138425136</v>
+        <v>38.25878415950206</v>
       </c>
       <c r="K2" t="n">
-        <v>35.60459462989069</v>
+        <v>36.5421642203677</v>
       </c>
       <c r="L2" t="n">
-        <v>27.99633849627728</v>
+        <v>33.40705642906815</v>
       </c>
     </row>
   </sheetData>
@@ -1950,37 +1950,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6967688750009984</v>
+        <v>147.0008939169929</v>
       </c>
       <c r="C2" t="n">
-        <v>41.18320409305016</v>
+        <v>48.37539854975108</v>
       </c>
       <c r="D2" t="n">
-        <v>34.49135943431597</v>
+        <v>47.65259828369323</v>
       </c>
       <c r="E2" t="n">
-        <v>50.69228584559489</v>
+        <v>53.87179269157685</v>
       </c>
       <c r="F2" t="n">
-        <v>37.77987671327077</v>
+        <v>45.32937821806353</v>
       </c>
       <c r="G2" t="n">
-        <v>39.11818594136139</v>
+        <v>56.97021057071613</v>
       </c>
       <c r="H2" t="n">
-        <v>42.94168810477329</v>
+        <v>49.71331862530472</v>
       </c>
       <c r="I2" t="n">
-        <v>50.53246703809751</v>
+        <v>56.17614727528404</v>
       </c>
       <c r="J2" t="n">
-        <v>38.59255878103754</v>
+        <v>43.70624065545719</v>
       </c>
       <c r="K2" t="n">
-        <v>52.71542474895082</v>
+        <v>52.79691463285969</v>
       </c>
       <c r="L2" t="n">
-        <v>41.94258067408273</v>
+        <v>43.35494963759501</v>
       </c>
     </row>
   </sheetData>
@@ -2064,37 +2064,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.706249916984234</v>
+        <v>141.4918934580055</v>
       </c>
       <c r="C2" t="n">
-        <v>43.32887710203971</v>
+        <v>54.43226035155814</v>
       </c>
       <c r="D2" t="n">
-        <v>38.63686341516248</v>
+        <v>53.23651680520622</v>
       </c>
       <c r="E2" t="n">
-        <v>47.20770749623724</v>
+        <v>47.54380661483028</v>
       </c>
       <c r="F2" t="n">
-        <v>33.54010786108915</v>
+        <v>33.96430859984829</v>
       </c>
       <c r="G2" t="n">
-        <v>42.74296212325605</v>
+        <v>43.21521548631198</v>
       </c>
       <c r="H2" t="n">
-        <v>44.54826177595782</v>
+        <v>44.46139588081177</v>
       </c>
       <c r="I2" t="n">
-        <v>43.42012296161482</v>
+        <v>45.64957194890849</v>
       </c>
       <c r="J2" t="n">
-        <v>39.60293149772233</v>
+        <v>42.20082754407338</v>
       </c>
       <c r="K2" t="n">
-        <v>36.54991203686053</v>
+        <v>45.24521244320095</v>
       </c>
       <c r="L2" t="n">
-        <v>51.95711855319546</v>
+        <v>52.50718864919871</v>
       </c>
     </row>
   </sheetData>
@@ -2178,34 +2178,34 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7080916669801809</v>
+        <v>137.707884708012</v>
       </c>
       <c r="C2" t="n">
-        <v>47.55265116166088</v>
+        <v>52.26142610534777</v>
       </c>
       <c r="D2" t="n">
         <v>44.34945197671834</v>
       </c>
       <c r="E2" t="n">
-        <v>43.70081365728223</v>
+        <v>48.68128501701714</v>
       </c>
       <c r="F2" t="n">
-        <v>39.26377775540449</v>
+        <v>50.43681485242693</v>
       </c>
       <c r="G2" t="n">
-        <v>36.06422760883811</v>
+        <v>42.60266685564086</v>
       </c>
       <c r="H2" t="n">
-        <v>41.71409737352798</v>
+        <v>47.60668022076609</v>
       </c>
       <c r="I2" t="n">
-        <v>30.73143544266909</v>
+        <v>32.36196743877598</v>
       </c>
       <c r="J2" t="n">
-        <v>39.08765418596403</v>
+        <v>43.84367594107773</v>
       </c>
       <c r="K2" t="n">
-        <v>63.46710030169166</v>
+        <v>64.38377501445001</v>
       </c>
       <c r="L2" t="n">
         <v>41.79392144507622</v>
@@ -2292,37 +2292,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7329865000210702</v>
+        <v>142.1550604170188</v>
       </c>
       <c r="C2" t="n">
-        <v>44.87970561862215</v>
+        <v>51.67647757010842</v>
       </c>
       <c r="D2" t="n">
-        <v>61.41345408726418</v>
+        <v>62.17164640381306</v>
       </c>
       <c r="E2" t="n">
         <v>30.96859011896896</v>
       </c>
       <c r="F2" t="n">
-        <v>35.97613361027557</v>
+        <v>41.26897081567744</v>
       </c>
       <c r="G2" t="n">
-        <v>33.96720590125854</v>
+        <v>39.07850261376875</v>
       </c>
       <c r="H2" t="n">
-        <v>44.70060943545036</v>
+        <v>44.91808798044719</v>
       </c>
       <c r="I2" t="n">
-        <v>38.89580248737084</v>
+        <v>43.47494587819795</v>
       </c>
       <c r="J2" t="n">
-        <v>49.85863443347831</v>
+        <v>52.22694981773388</v>
       </c>
       <c r="K2" t="n">
-        <v>41.5457699529143</v>
+        <v>52.83345162007875</v>
       </c>
       <c r="L2" t="n">
-        <v>32.61939587263073</v>
+        <v>37.3295064469383</v>
       </c>
     </row>
   </sheetData>
@@ -2406,37 +2406,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6934338749852031</v>
+        <v>139.775180458033</v>
       </c>
       <c r="C2" t="n">
-        <v>57.07604250970104</v>
+        <v>57.66940156917713</v>
       </c>
       <c r="D2" t="n">
-        <v>34.5851294651717</v>
+        <v>49.30963310863361</v>
       </c>
       <c r="E2" t="n">
         <v>51.3496291333423</v>
       </c>
       <c r="F2" t="n">
-        <v>39.3162900344244</v>
+        <v>48.28254408333996</v>
       </c>
       <c r="G2" t="n">
-        <v>32.24173925768895</v>
+        <v>34.86649481922792</v>
       </c>
       <c r="H2" t="n">
-        <v>43.20058940814253</v>
+        <v>43.24958921164709</v>
       </c>
       <c r="I2" t="n">
-        <v>51.05090080019556</v>
+        <v>52.04279841656315</v>
       </c>
       <c r="J2" t="n">
-        <v>53.27082668443169</v>
+        <v>52.75616549940197</v>
       </c>
       <c r="K2" t="n">
-        <v>36.48168932890555</v>
+        <v>36.27956331112553</v>
       </c>
       <c r="L2" t="n">
-        <v>42.41005439158444</v>
+        <v>42.9681368604683</v>
       </c>
     </row>
   </sheetData>
@@ -2520,37 +2520,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7132465409813449</v>
+        <v>138.8029046250158</v>
       </c>
       <c r="C2" t="n">
-        <v>41.50554175397161</v>
+        <v>41.43006494404842</v>
       </c>
       <c r="D2" t="n">
-        <v>47.73866527886594</v>
+        <v>50.09925488495853</v>
       </c>
       <c r="E2" t="n">
         <v>37.40709306412095</v>
       </c>
       <c r="F2" t="n">
-        <v>41.78619934203246</v>
+        <v>42.39451522949106</v>
       </c>
       <c r="G2" t="n">
-        <v>32.4238715065986</v>
+        <v>36.70369177352181</v>
       </c>
       <c r="H2" t="n">
-        <v>60.72251266542179</v>
+        <v>61.28018298433721</v>
       </c>
       <c r="I2" t="n">
-        <v>34.22347316725659</v>
+        <v>43.83563081715869</v>
       </c>
       <c r="J2" t="n">
-        <v>42.51698384279597</v>
+        <v>41.41296927246946</v>
       </c>
       <c r="K2" t="n">
-        <v>45.61061444860373</v>
+        <v>45.4154548306945</v>
       </c>
       <c r="L2" t="n">
-        <v>44.45951644811851</v>
+        <v>45.24094696566749</v>
       </c>
     </row>
   </sheetData>
@@ -2634,37 +2634,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6727607080247253</v>
+        <v>136.8439691250096</v>
       </c>
       <c r="C2" t="n">
-        <v>38.1881225621783</v>
+        <v>43.54532106487185</v>
       </c>
       <c r="D2" t="n">
-        <v>37.54435367253856</v>
+        <v>37.62629048496451</v>
       </c>
       <c r="E2" t="n">
-        <v>41.48019946353926</v>
+        <v>46.24545336479803</v>
       </c>
       <c r="F2" t="n">
-        <v>37.4799338092614</v>
+        <v>37.47330600322829</v>
       </c>
       <c r="G2" t="n">
-        <v>43.47136975753605</v>
+        <v>46.68808330192601</v>
       </c>
       <c r="H2" t="n">
-        <v>53.45878816513264</v>
+        <v>53.4286189555377</v>
       </c>
       <c r="I2" t="n">
-        <v>36.09821228425663</v>
+        <v>45.48955454916115</v>
       </c>
       <c r="J2" t="n">
-        <v>39.20042227524115</v>
+        <v>39.65831183888007</v>
       </c>
       <c r="K2" t="n">
-        <v>46.19420679096792</v>
+        <v>49.18041479178285</v>
       </c>
       <c r="L2" t="n">
-        <v>30.50232014221784</v>
+        <v>30.59237590422887</v>
       </c>
     </row>
   </sheetData>
@@ -2748,37 +2748,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6742180000292137</v>
+        <v>137.163034749974</v>
       </c>
       <c r="C2" t="n">
-        <v>50.9305851964066</v>
+        <v>52.02831190051816</v>
       </c>
       <c r="D2" t="n">
-        <v>37.95935514269348</v>
+        <v>44.61041672325588</v>
       </c>
       <c r="E2" t="n">
-        <v>58.46255519306365</v>
+        <v>59.31278734845294</v>
       </c>
       <c r="F2" t="n">
         <v>24.49680049380828</v>
       </c>
       <c r="G2" t="n">
-        <v>55.45464774395306</v>
+        <v>55.29380383987952</v>
       </c>
       <c r="H2" t="n">
-        <v>39.3619124626521</v>
+        <v>49.05567808420189</v>
       </c>
       <c r="I2" t="n">
-        <v>38.20312918061266</v>
+        <v>46.58035652343062</v>
       </c>
       <c r="J2" t="n">
-        <v>35.22148531576916</v>
+        <v>41.13306949568204</v>
       </c>
       <c r="K2" t="n">
-        <v>36.46275477131196</v>
+        <v>40.88051409007619</v>
       </c>
       <c r="L2" t="n">
-        <v>35.12172501303346</v>
+        <v>35.42047999707508</v>
       </c>
     </row>
   </sheetData>
@@ -2862,34 +2862,34 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6658685840084217</v>
+        <v>137.1576854159939</v>
       </c>
       <c r="C2" t="n">
-        <v>37.76446520344778</v>
+        <v>44.51862642488238</v>
       </c>
       <c r="D2" t="n">
-        <v>49.83776858115197</v>
+        <v>63.1880830593269</v>
       </c>
       <c r="E2" t="n">
-        <v>38.21975911116076</v>
+        <v>42.97137406522848</v>
       </c>
       <c r="F2" t="n">
-        <v>35.73950622104421</v>
+        <v>42.9597914449851</v>
       </c>
       <c r="G2" t="n">
-        <v>40.49591054109781</v>
+        <v>40.92829123616117</v>
       </c>
       <c r="H2" t="n">
-        <v>37.97953851066968</v>
+        <v>38.87680584729788</v>
       </c>
       <c r="I2" t="n">
-        <v>39.37674772905704</v>
+        <v>48.59239917108244</v>
       </c>
       <c r="J2" t="n">
-        <v>47.97427363926052</v>
+        <v>52.4401247948505</v>
       </c>
       <c r="K2" t="n">
-        <v>33.4154735167834</v>
+        <v>34.3796058273337</v>
       </c>
       <c r="L2" t="n">
         <v>30.03343075985319</v>
@@ -2976,37 +2976,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7091141249984503</v>
+        <v>140.6823012499954</v>
       </c>
       <c r="C2" t="n">
-        <v>66.6448852652286</v>
+        <v>66.66614311742161</v>
       </c>
       <c r="D2" t="n">
-        <v>41.66722581597411</v>
+        <v>38.82812001972982</v>
       </c>
       <c r="E2" t="n">
-        <v>46.45470669497135</v>
+        <v>60.10434682772627</v>
       </c>
       <c r="F2" t="n">
-        <v>41.92713919642183</v>
+        <v>42.46451474449447</v>
       </c>
       <c r="G2" t="n">
-        <v>31.86723793554827</v>
+        <v>31.7419501369602</v>
       </c>
       <c r="H2" t="n">
         <v>37.79108922656612</v>
       </c>
       <c r="I2" t="n">
-        <v>38.91057758539123</v>
+        <v>39.19380748889014</v>
       </c>
       <c r="J2" t="n">
-        <v>40.4493487662286</v>
+        <v>44.71363236414593</v>
       </c>
       <c r="K2" t="n">
-        <v>48.58683605428232</v>
+        <v>51.87708636285332</v>
       </c>
       <c r="L2" t="n">
-        <v>35.45136333713052</v>
+        <v>44.09914587203605</v>
       </c>
     </row>
   </sheetData>
@@ -3090,37 +3090,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6629935000091791</v>
+        <v>134.0286194159999</v>
       </c>
       <c r="C2" t="n">
-        <v>34.44645559132724</v>
+        <v>38.31010913695528</v>
       </c>
       <c r="D2" t="n">
-        <v>30.71378620624894</v>
+        <v>34.4248701043299</v>
       </c>
       <c r="E2" t="n">
         <v>41.96945867359436</v>
       </c>
       <c r="F2" t="n">
-        <v>31.35316246321928</v>
+        <v>39.106740239758</v>
       </c>
       <c r="G2" t="n">
-        <v>49.10429900430706</v>
+        <v>49.9070906272583</v>
       </c>
       <c r="H2" t="n">
-        <v>41.65670511294064</v>
+        <v>41.56578783479479</v>
       </c>
       <c r="I2" t="n">
-        <v>38.86605824455729</v>
+        <v>38.74053659264091</v>
       </c>
       <c r="J2" t="n">
-        <v>42.19253479439337</v>
+        <v>44.9786899331033</v>
       </c>
       <c r="K2" t="n">
-        <v>54.10130310391623</v>
+        <v>49.27561375799898</v>
       </c>
       <c r="L2" t="n">
-        <v>31.30635588416547</v>
+        <v>32.72331883944486</v>
       </c>
     </row>
   </sheetData>
@@ -3204,37 +3204,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8961369580356404</v>
+        <v>140.6853640420013</v>
       </c>
       <c r="C2" t="n">
-        <v>41.52670062247953</v>
+        <v>41.85314491880742</v>
       </c>
       <c r="D2" t="n">
-        <v>40.46584573505485</v>
+        <v>46.78683784506823</v>
       </c>
       <c r="E2" t="n">
-        <v>45.64085607223861</v>
+        <v>51.73312929796241</v>
       </c>
       <c r="F2" t="n">
-        <v>36.69206005840376</v>
+        <v>35.99133598137816</v>
       </c>
       <c r="G2" t="n">
-        <v>22.59455323383089</v>
+        <v>22.81677468348914</v>
       </c>
       <c r="H2" t="n">
-        <v>49.52596870900369</v>
+        <v>49.90458167684238</v>
       </c>
       <c r="I2" t="n">
-        <v>49.60105318157153</v>
+        <v>52.87559796989618</v>
       </c>
       <c r="J2" t="n">
-        <v>46.99272608838751</v>
+        <v>47.12756589908498</v>
       </c>
       <c r="K2" t="n">
-        <v>50.38257382979712</v>
+        <v>57.18668045639778</v>
       </c>
       <c r="L2" t="n">
-        <v>35.19375452570804</v>
+        <v>44.57543182894069</v>
       </c>
     </row>
   </sheetData>
@@ -3318,37 +3318,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6841318749939092</v>
+        <v>137.6656791669666</v>
       </c>
       <c r="C2" t="n">
-        <v>38.30988704564602</v>
+        <v>43.17820704188696</v>
       </c>
       <c r="D2" t="n">
-        <v>32.96836377913294</v>
+        <v>38.54099017787227</v>
       </c>
       <c r="E2" t="n">
-        <v>50.99079254758629</v>
+        <v>51.48830753290013</v>
       </c>
       <c r="F2" t="n">
-        <v>50.93195422579562</v>
+        <v>51.24511258942992</v>
       </c>
       <c r="G2" t="n">
-        <v>45.98618843837149</v>
+        <v>49.35216035660603</v>
       </c>
       <c r="H2" t="n">
         <v>46.30035788636026</v>
       </c>
       <c r="I2" t="n">
-        <v>42.38756965293836</v>
+        <v>45.48235453980904</v>
       </c>
       <c r="J2" t="n">
-        <v>31.85657539359903</v>
+        <v>35.8280236444241</v>
       </c>
       <c r="K2" t="n">
-        <v>41.23520167750516</v>
+        <v>40.89716257323172</v>
       </c>
       <c r="L2" t="n">
-        <v>42.32770600562003</v>
+        <v>45.47435609541111</v>
       </c>
     </row>
   </sheetData>
@@ -3432,37 +3432,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6778923330130056</v>
+        <v>136.8340540830395</v>
       </c>
       <c r="C2" t="n">
-        <v>42.67375249952514</v>
+        <v>43.82160536017182</v>
       </c>
       <c r="D2" t="n">
         <v>52.08920801517548</v>
       </c>
       <c r="E2" t="n">
-        <v>31.89084583006079</v>
+        <v>37.50658583811985</v>
       </c>
       <c r="F2" t="n">
-        <v>47.21877190326821</v>
+        <v>53.32474269443582</v>
       </c>
       <c r="G2" t="n">
-        <v>46.66365921269258</v>
+        <v>46.25693551886733</v>
       </c>
       <c r="H2" t="n">
-        <v>38.89936226188642</v>
+        <v>44.27150834773474</v>
       </c>
       <c r="I2" t="n">
-        <v>41.10934002328008</v>
+        <v>43.29220687337599</v>
       </c>
       <c r="J2" t="n">
-        <v>55.22812514697094</v>
+        <v>57.72430234316897</v>
       </c>
       <c r="K2" t="n">
-        <v>34.29787028552391</v>
+        <v>43.60126355016732</v>
       </c>
       <c r="L2" t="n">
-        <v>31.76027863695827</v>
+        <v>31.792814418491</v>
       </c>
     </row>
   </sheetData>
@@ -3546,25 +3546,25 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6421040419954807</v>
+        <v>132.0462053330266</v>
       </c>
       <c r="C2" t="n">
-        <v>30.8345876888616</v>
+        <v>38.55210564784149</v>
       </c>
       <c r="D2" t="n">
-        <v>29.68267134085984</v>
+        <v>35.76749322306015</v>
       </c>
       <c r="E2" t="n">
-        <v>40.83689291099758</v>
+        <v>41.31587706215162</v>
       </c>
       <c r="F2" t="n">
-        <v>44.12247261922227</v>
+        <v>44.42391464236236</v>
       </c>
       <c r="G2" t="n">
-        <v>44.89616232252946</v>
+        <v>43.53823251023225</v>
       </c>
       <c r="H2" t="n">
-        <v>33.18929366277444</v>
+        <v>33.31750322026275</v>
       </c>
       <c r="I2" t="n">
         <v>27.23226658161643</v>
@@ -3573,10 +3573,10 @@
         <v>32.27850944728133</v>
       </c>
       <c r="K2" t="n">
-        <v>57.14774517894593</v>
+        <v>67.08066928262321</v>
       </c>
       <c r="L2" t="n">
-        <v>35.23982491128792</v>
+        <v>39.26988003411579</v>
       </c>
     </row>
   </sheetData>
@@ -3660,37 +3660,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6284043330233544</v>
+        <v>126.303456124966</v>
       </c>
       <c r="C2" t="n">
-        <v>42.31109958967303</v>
+        <v>48.4873226777058</v>
       </c>
       <c r="D2" t="n">
-        <v>58.08792247251557</v>
+        <v>58.83085944647058</v>
       </c>
       <c r="E2" t="n">
-        <v>47.74588904207773</v>
+        <v>47.76706209152439</v>
       </c>
       <c r="F2" t="n">
-        <v>35.40103872674094</v>
+        <v>36.14620833883776</v>
       </c>
       <c r="G2" t="n">
-        <v>34.91781858717217</v>
+        <v>48.31488115236625</v>
       </c>
       <c r="H2" t="n">
-        <v>54.75595362724132</v>
+        <v>58.17299981154891</v>
       </c>
       <c r="I2" t="n">
-        <v>44.31893374627396</v>
+        <v>44.67747671757878</v>
       </c>
       <c r="J2" t="n">
-        <v>34.88385795462582</v>
+        <v>34.89146243955634</v>
       </c>
       <c r="K2" t="n">
-        <v>39.80967553040641</v>
+        <v>39.54115502415128</v>
       </c>
       <c r="L2" t="n">
-        <v>27.67628761457252</v>
+        <v>30.37521802442591</v>
       </c>
     </row>
   </sheetData>
@@ -3774,37 +3774,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6897254170035012</v>
+        <v>135.0310596250347</v>
       </c>
       <c r="C2" t="n">
-        <v>41.90960064908728</v>
+        <v>42.02304196857281</v>
       </c>
       <c r="D2" t="n">
-        <v>42.35278374369572</v>
+        <v>45.05186354835476</v>
       </c>
       <c r="E2" t="n">
-        <v>43.56616899705371</v>
+        <v>43.73440505087176</v>
       </c>
       <c r="F2" t="n">
         <v>30.32962239032873</v>
       </c>
       <c r="G2" t="n">
-        <v>39.32027972199376</v>
+        <v>39.76141604737771</v>
       </c>
       <c r="H2" t="n">
-        <v>47.47220581852513</v>
+        <v>47.85947078658504</v>
       </c>
       <c r="I2" t="n">
-        <v>44.50361940912278</v>
+        <v>48.43195761361133</v>
       </c>
       <c r="J2" t="n">
-        <v>39.24141323803062</v>
+        <v>40.08633419418332</v>
       </c>
       <c r="K2" t="n">
-        <v>58.74268420634078</v>
+        <v>60.19036250549726</v>
       </c>
       <c r="L2" t="n">
-        <v>35.31853068197643</v>
+        <v>38.5495109953473</v>
       </c>
     </row>
   </sheetData>
@@ -3888,37 +3888,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6460309580434114</v>
+        <v>133.9901323340018</v>
       </c>
       <c r="C2" t="n">
-        <v>33.02562595343392</v>
+        <v>32.9384891572297</v>
       </c>
       <c r="D2" t="n">
-        <v>42.83705296543891</v>
+        <v>43.11323498471495</v>
       </c>
       <c r="E2" t="n">
-        <v>42.44702031143783</v>
+        <v>44.03760364702966</v>
       </c>
       <c r="F2" t="n">
-        <v>32.28454274145985</v>
+        <v>36.64202283333447</v>
       </c>
       <c r="G2" t="n">
-        <v>45.67640698611427</v>
+        <v>45.70175026463237</v>
       </c>
       <c r="H2" t="n">
-        <v>50.5240910304714</v>
+        <v>50.70229192975624</v>
       </c>
       <c r="I2" t="n">
         <v>38.79020775609448</v>
       </c>
       <c r="J2" t="n">
-        <v>57.54480431045145</v>
+        <v>61.04269942795089</v>
       </c>
       <c r="K2" t="n">
-        <v>31.44541599867215</v>
+        <v>35.38662126588731</v>
       </c>
       <c r="L2" t="n">
-        <v>28.87882974946213</v>
+        <v>40.87160553716254</v>
       </c>
     </row>
   </sheetData>
@@ -4002,37 +4002,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.666388250014279</v>
+        <v>139.9804715829669</v>
       </c>
       <c r="C2" t="n">
-        <v>35.42252017201852</v>
+        <v>41.01494064824323</v>
       </c>
       <c r="D2" t="n">
-        <v>56.65984274800587</v>
+        <v>55.51069208653486</v>
       </c>
       <c r="E2" t="n">
-        <v>50.04258378350266</v>
+        <v>54.21630863541354</v>
       </c>
       <c r="F2" t="n">
-        <v>38.79328804617992</v>
+        <v>43.48410491026821</v>
       </c>
       <c r="G2" t="n">
-        <v>26.6591953934009</v>
+        <v>30.68157547163331</v>
       </c>
       <c r="H2" t="n">
-        <v>37.50707048128518</v>
+        <v>41.68816712972068</v>
       </c>
       <c r="I2" t="n">
-        <v>47.35684973754703</v>
+        <v>47.5271688868915</v>
       </c>
       <c r="J2" t="n">
-        <v>61.29663661645674</v>
+        <v>62.11939034636224</v>
       </c>
       <c r="K2" t="n">
-        <v>41.68093463441936</v>
+        <v>45.11876065246942</v>
       </c>
       <c r="L2" t="n">
-        <v>49.64465434826117</v>
+        <v>54.53814766386814</v>
       </c>
     </row>
   </sheetData>
@@ -4116,37 +4116,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6740397920366377</v>
+        <v>148.6922674169764</v>
       </c>
       <c r="C2" t="n">
         <v>48.72905909381089</v>
       </c>
       <c r="D2" t="n">
-        <v>45.8107744798598</v>
+        <v>48.10646137872448</v>
       </c>
       <c r="E2" t="n">
-        <v>47.4397468167701</v>
+        <v>51.00249964378183</v>
       </c>
       <c r="F2" t="n">
-        <v>30.49579555862159</v>
+        <v>33.98191427107297</v>
       </c>
       <c r="G2" t="n">
-        <v>58.20853329982376</v>
+        <v>61.8750621663208</v>
       </c>
       <c r="H2" t="n">
-        <v>47.33120913550767</v>
+        <v>47.79281257147034</v>
       </c>
       <c r="I2" t="n">
-        <v>34.56051148369522</v>
+        <v>34.47288311840654</v>
       </c>
       <c r="J2" t="n">
-        <v>36.36976305838174</v>
+        <v>47.05848377998343</v>
       </c>
       <c r="K2" t="n">
         <v>50.58263197984496</v>
       </c>
       <c r="L2" t="n">
-        <v>51.45532701952381</v>
+        <v>55.9266010898201</v>
       </c>
     </row>
   </sheetData>
@@ -4230,37 +4230,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6666075420216657</v>
+        <v>144.5313121659565</v>
       </c>
       <c r="C2" t="n">
-        <v>44.29317278101465</v>
+        <v>49.35179628324205</v>
       </c>
       <c r="D2" t="n">
-        <v>44.39161850993096</v>
+        <v>44.82179508946217</v>
       </c>
       <c r="E2" t="n">
-        <v>26.87422709099512</v>
+        <v>34.22593677026423</v>
       </c>
       <c r="F2" t="n">
-        <v>31.52138387667755</v>
+        <v>37.39306113832495</v>
       </c>
       <c r="G2" t="n">
-        <v>50.80140879484367</v>
+        <v>51.22765759566813</v>
       </c>
       <c r="H2" t="n">
-        <v>55.62257349269791</v>
+        <v>55.46992853075966</v>
       </c>
       <c r="I2" t="n">
-        <v>52.90482563720764</v>
+        <v>52.29987503010817</v>
       </c>
       <c r="J2" t="n">
-        <v>46.15598292303221</v>
+        <v>45.66401528597753</v>
       </c>
       <c r="K2" t="n">
-        <v>41.19650028536795</v>
+        <v>48.43677786394935</v>
       </c>
       <c r="L2" t="n">
-        <v>41.74909572038849</v>
+        <v>42.90625105325428</v>
       </c>
     </row>
   </sheetData>
@@ -4344,37 +4344,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6797591249924153</v>
+        <v>147.5032400830532</v>
       </c>
       <c r="C2" t="n">
-        <v>38.05648999281414</v>
+        <v>40.44071998221588</v>
       </c>
       <c r="D2" t="n">
-        <v>29.93098156218627</v>
+        <v>30.39577876064064</v>
       </c>
       <c r="E2" t="n">
-        <v>38.80701902565836</v>
+        <v>39.04027881325828</v>
       </c>
       <c r="F2" t="n">
-        <v>49.68289931653209</v>
+        <v>56.12300404092493</v>
       </c>
       <c r="G2" t="n">
-        <v>37.81177460626618</v>
+        <v>49.62141170899037</v>
       </c>
       <c r="H2" t="n">
-        <v>47.39628421309137</v>
+        <v>51.10908859675517</v>
       </c>
       <c r="I2" t="n">
-        <v>50.11511037953991</v>
+        <v>52.30201542991191</v>
       </c>
       <c r="J2" t="n">
-        <v>36.9166301347731</v>
+        <v>42.33791520264938</v>
       </c>
       <c r="K2" t="n">
-        <v>35.72710126773632</v>
+        <v>37.09436990568187</v>
       </c>
       <c r="L2" t="n">
-        <v>37.94715871931582</v>
+        <v>43.2216209978446</v>
       </c>
     </row>
   </sheetData>
@@ -4458,37 +4458,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7428059169906192</v>
+        <v>143.9223024169914</v>
       </c>
       <c r="C2" t="n">
-        <v>46.43117470620491</v>
+        <v>46.347742950297</v>
       </c>
       <c r="D2" t="n">
-        <v>44.29640558289621</v>
+        <v>46.43411165585781</v>
       </c>
       <c r="E2" t="n">
-        <v>34.84654785899992</v>
+        <v>34.14462172021904</v>
       </c>
       <c r="F2" t="n">
-        <v>40.79865296642177</v>
+        <v>43.54583088352603</v>
       </c>
       <c r="G2" t="n">
-        <v>31.3029982618174</v>
+        <v>36.27143613407908</v>
       </c>
       <c r="H2" t="n">
-        <v>37.08686055081219</v>
+        <v>37.24902385412204</v>
       </c>
       <c r="I2" t="n">
-        <v>33.22284605361004</v>
+        <v>42.24704556485356</v>
       </c>
       <c r="J2" t="n">
-        <v>37.33744353087073</v>
+        <v>37.54023512054278</v>
       </c>
       <c r="K2" t="n">
         <v>36.58243823999828</v>
       </c>
       <c r="L2" t="n">
-        <v>37.86844096939616</v>
+        <v>41.96201580141906</v>
       </c>
     </row>
   </sheetData>
@@ -4572,34 +4572,34 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.664441832981538</v>
+        <v>145.3355955409934</v>
       </c>
       <c r="C2" t="n">
-        <v>35.58264557310182</v>
+        <v>42.12344161472293</v>
       </c>
       <c r="D2" t="n">
-        <v>37.13331240092531</v>
+        <v>42.08002278396463</v>
       </c>
       <c r="E2" t="n">
-        <v>42.42207336458763</v>
+        <v>42.03063472988652</v>
       </c>
       <c r="F2" t="n">
-        <v>52.54619409542003</v>
+        <v>56.10308595783653</v>
       </c>
       <c r="G2" t="n">
-        <v>38.35861822600649</v>
+        <v>51.71175541223243</v>
       </c>
       <c r="H2" t="n">
         <v>30.47364295819383</v>
       </c>
       <c r="I2" t="n">
-        <v>33.27041192467566</v>
+        <v>33.48978475261949</v>
       </c>
       <c r="J2" t="n">
-        <v>40.58645357813954</v>
+        <v>52.61271902276765</v>
       </c>
       <c r="K2" t="n">
-        <v>31.51761271717516</v>
+        <v>35.4220491565876</v>
       </c>
       <c r="L2" t="n">
         <v>49.32532034558569</v>
@@ -4686,22 +4686,22 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6634491250151768</v>
+        <v>147.3799726659781</v>
       </c>
       <c r="C2" t="n">
-        <v>39.01811320789328</v>
+        <v>47.24966456650399</v>
       </c>
       <c r="D2" t="n">
-        <v>32.9833384692912</v>
+        <v>37.09308323779748</v>
       </c>
       <c r="E2" t="n">
-        <v>36.67785535550687</v>
+        <v>36.29748064480717</v>
       </c>
       <c r="F2" t="n">
-        <v>23.04917695484936</v>
+        <v>22.9198775891988</v>
       </c>
       <c r="G2" t="n">
-        <v>44.30287224573168</v>
+        <v>49.93192136651425</v>
       </c>
       <c r="H2" t="n">
         <v>51.09828356902336</v>
@@ -4710,10 +4710,10 @@
         <v>50.8003216126309</v>
       </c>
       <c r="J2" t="n">
-        <v>45.6611783983313</v>
+        <v>47.9642025653466</v>
       </c>
       <c r="K2" t="n">
-        <v>44.83887971190423</v>
+        <v>50.49055871440487</v>
       </c>
       <c r="L2" t="n">
         <v>47.24053637438332</v>
@@ -4800,37 +4800,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6876572080072947</v>
+        <v>155.4348979999777</v>
       </c>
       <c r="C2" t="n">
-        <v>32.8323886868599</v>
+        <v>38.89192761516671</v>
       </c>
       <c r="D2" t="n">
-        <v>47.13427937010077</v>
+        <v>52.36504311923359</v>
       </c>
       <c r="E2" t="n">
-        <v>52.14017285713685</v>
+        <v>51.67310549511877</v>
       </c>
       <c r="F2" t="n">
-        <v>36.43314958740626</v>
+        <v>43.07262106250043</v>
       </c>
       <c r="G2" t="n">
-        <v>29.60151381778573</v>
+        <v>35.68433102525184</v>
       </c>
       <c r="H2" t="n">
-        <v>43.02890919133417</v>
+        <v>45.50751692281946</v>
       </c>
       <c r="I2" t="n">
-        <v>49.88778793618841</v>
+        <v>49.8338071763261</v>
       </c>
       <c r="J2" t="n">
-        <v>48.66514956762794</v>
+        <v>46.54073707078769</v>
       </c>
       <c r="K2" t="n">
-        <v>39.5355981628276</v>
+        <v>43.85053321969752</v>
       </c>
       <c r="L2" t="n">
-        <v>44.67241143098216</v>
+        <v>52.24734431776344</v>
       </c>
     </row>
   </sheetData>
@@ -4914,37 +4914,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.649883583013434</v>
+        <v>155.0001601660042</v>
       </c>
       <c r="C2" t="n">
-        <v>43.25364590357398</v>
+        <v>43.33283905461434</v>
       </c>
       <c r="D2" t="n">
-        <v>31.81089825306026</v>
+        <v>36.45223378706292</v>
       </c>
       <c r="E2" t="n">
-        <v>46.03463827760253</v>
+        <v>53.77210227214868</v>
       </c>
       <c r="F2" t="n">
-        <v>37.45418764899127</v>
+        <v>37.2736903405621</v>
       </c>
       <c r="G2" t="n">
-        <v>46.22349189209655</v>
+        <v>45.46131193922361</v>
       </c>
       <c r="H2" t="n">
-        <v>40.02754149607546</v>
+        <v>39.69492413738008</v>
       </c>
       <c r="I2" t="n">
-        <v>39.17143820520212</v>
+        <v>39.01045709322052</v>
       </c>
       <c r="J2" t="n">
-        <v>28.03993261468443</v>
+        <v>32.50736380176453</v>
       </c>
       <c r="K2" t="n">
-        <v>30.54621786815423</v>
+        <v>35.38433881838519</v>
       </c>
       <c r="L2" t="n">
-        <v>35.26545122760446</v>
+        <v>37.83495329776365</v>
       </c>
     </row>
   </sheetData>
@@ -5028,37 +5028,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6723009999841452</v>
+        <v>145.8679649580154</v>
       </c>
       <c r="C2" t="n">
-        <v>32.71345461012002</v>
+        <v>34.49083869898745</v>
       </c>
       <c r="D2" t="n">
-        <v>30.44781911091724</v>
+        <v>30.45569942126519</v>
       </c>
       <c r="E2" t="n">
-        <v>44.20065061490735</v>
+        <v>55.15785057159931</v>
       </c>
       <c r="F2" t="n">
-        <v>44.11622071070953</v>
+        <v>44.69212184927254</v>
       </c>
       <c r="G2" t="n">
-        <v>34.3944506128221</v>
+        <v>43.6676176844127</v>
       </c>
       <c r="H2" t="n">
-        <v>39.17564922686081</v>
+        <v>44.74438704780437</v>
       </c>
       <c r="I2" t="n">
-        <v>39.27477978248981</v>
+        <v>40.10002479757486</v>
       </c>
       <c r="J2" t="n">
-        <v>41.34715688028319</v>
+        <v>41.6652700718053</v>
       </c>
       <c r="K2" t="n">
-        <v>36.61553117271718</v>
+        <v>39.97704320681049</v>
       </c>
       <c r="L2" t="n">
-        <v>41.3876267310095</v>
+        <v>45.02739696756751</v>
       </c>
     </row>
   </sheetData>
@@ -5142,37 +5142,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6969556250260212</v>
+        <v>152.8601063750102</v>
       </c>
       <c r="C2" t="n">
-        <v>35.70535836605781</v>
+        <v>42.32299213561907</v>
       </c>
       <c r="D2" t="n">
-        <v>39.29862409172831</v>
+        <v>49.5820616673246</v>
       </c>
       <c r="E2" t="n">
-        <v>38.5983597210999</v>
+        <v>38.64615828014495</v>
       </c>
       <c r="F2" t="n">
-        <v>45.46257787344462</v>
+        <v>49.5230593276853</v>
       </c>
       <c r="G2" t="n">
-        <v>40.54807275106901</v>
+        <v>43.32055737486276</v>
       </c>
       <c r="H2" t="n">
-        <v>25.1486907078257</v>
+        <v>30.41655861409425</v>
       </c>
       <c r="I2" t="n">
-        <v>42.29347147943715</v>
+        <v>40.92780798130687</v>
       </c>
       <c r="J2" t="n">
-        <v>37.00607421486438</v>
+        <v>45.00746952124614</v>
       </c>
       <c r="K2" t="n">
-        <v>40.89870742576558</v>
+        <v>45.34646953531733</v>
       </c>
       <c r="L2" t="n">
-        <v>43.32972238242201</v>
+        <v>42.72908280989898</v>
       </c>
     </row>
   </sheetData>
@@ -5256,37 +5256,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.709391999989748</v>
+        <v>158.0364964579931</v>
       </c>
       <c r="C2" t="n">
-        <v>41.23676990702923</v>
+        <v>43.72078504877803</v>
       </c>
       <c r="D2" t="n">
-        <v>48.26213381041058</v>
+        <v>50.15580019999577</v>
       </c>
       <c r="E2" t="n">
-        <v>57.92749919348</v>
+        <v>61.92827600538709</v>
       </c>
       <c r="F2" t="n">
-        <v>43.88150397796606</v>
+        <v>52.60064903320914</v>
       </c>
       <c r="G2" t="n">
-        <v>38.69195493646703</v>
+        <v>38.89165858480344</v>
       </c>
       <c r="H2" t="n">
-        <v>44.0835180549069</v>
+        <v>44.50704678439885</v>
       </c>
       <c r="I2" t="n">
-        <v>43.22001955303537</v>
+        <v>46.71239243559689</v>
       </c>
       <c r="J2" t="n">
-        <v>47.09902884248939</v>
+        <v>52.28324931581994</v>
       </c>
       <c r="K2" t="n">
-        <v>43.12782760227861</v>
+        <v>51.70191342164453</v>
       </c>
       <c r="L2" t="n">
-        <v>41.55655755869804</v>
+        <v>50.83079149524533</v>
       </c>
     </row>
   </sheetData>
@@ -5370,34 +5370,34 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6712543329922482</v>
+        <v>151.3440657500178</v>
       </c>
       <c r="C2" t="n">
-        <v>34.25693502927506</v>
+        <v>39.62717544662048</v>
       </c>
       <c r="D2" t="n">
-        <v>38.66608846761122</v>
+        <v>37.43045813537779</v>
       </c>
       <c r="E2" t="n">
-        <v>49.92547652358292</v>
+        <v>48.0143338607994</v>
       </c>
       <c r="F2" t="n">
-        <v>37.02218084010397</v>
+        <v>36.17841515055265</v>
       </c>
       <c r="G2" t="n">
-        <v>42.88501196526105</v>
+        <v>47.39735650458482</v>
       </c>
       <c r="H2" t="n">
         <v>41.12941418556612</v>
       </c>
       <c r="I2" t="n">
-        <v>32.26667413542926</v>
+        <v>36.45274335773939</v>
       </c>
       <c r="J2" t="n">
-        <v>43.62965279748504</v>
+        <v>43.56692547834121</v>
       </c>
       <c r="K2" t="n">
-        <v>33.0573220498616</v>
+        <v>33.12542549808392</v>
       </c>
       <c r="L2" t="n">
         <v>73.58473410426009</v>
@@ -5484,37 +5484,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6773715839954093</v>
+        <v>156.2581823330256</v>
       </c>
       <c r="C2" t="n">
-        <v>31.78334688730222</v>
+        <v>39.64333459692005</v>
       </c>
       <c r="D2" t="n">
-        <v>51.57993410570225</v>
+        <v>51.36519641505447</v>
       </c>
       <c r="E2" t="n">
-        <v>49.53050953686134</v>
+        <v>50.37091751331134</v>
       </c>
       <c r="F2" t="n">
-        <v>43.59591706341793</v>
+        <v>45.56656022280063</v>
       </c>
       <c r="G2" t="n">
-        <v>34.42540064535319</v>
+        <v>38.46764392879893</v>
       </c>
       <c r="H2" t="n">
-        <v>39.26338260469782</v>
+        <v>42.75231119421203</v>
       </c>
       <c r="I2" t="n">
-        <v>42.61016469782415</v>
+        <v>48.8745774893845</v>
       </c>
       <c r="J2" t="n">
-        <v>37.69273146833046</v>
+        <v>48.7625402602979</v>
       </c>
       <c r="K2" t="n">
-        <v>47.82728793031112</v>
+        <v>47.98220984727606</v>
       </c>
       <c r="L2" t="n">
-        <v>32.09987324510161</v>
+        <v>37.82838929143153</v>
       </c>
     </row>
   </sheetData>
@@ -5598,31 +5598,31 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6586876250221394</v>
+        <v>153.0010192919872</v>
       </c>
       <c r="C2" t="n">
-        <v>40.91712120160056</v>
+        <v>43.16479009966892</v>
       </c>
       <c r="D2" t="n">
-        <v>54.43075213195551</v>
+        <v>54.97975347942157</v>
       </c>
       <c r="E2" t="n">
-        <v>34.0558051531211</v>
+        <v>34.15967826871632</v>
       </c>
       <c r="F2" t="n">
-        <v>36.79721477690825</v>
+        <v>49.8962332031269</v>
       </c>
       <c r="G2" t="n">
-        <v>41.21588702173108</v>
+        <v>41.6126086201597</v>
       </c>
       <c r="H2" t="n">
-        <v>34.56513103598792</v>
+        <v>34.15812437397162</v>
       </c>
       <c r="I2" t="n">
-        <v>48.82861135562333</v>
+        <v>51.84851648119463</v>
       </c>
       <c r="J2" t="n">
-        <v>41.92209624000142</v>
+        <v>53.75091197580996</v>
       </c>
       <c r="K2" t="n">
         <v>43.83095491313285</v>
@@ -5712,37 +5712,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7086853749933653</v>
+        <v>144.7761631659814</v>
       </c>
       <c r="C2" t="n">
-        <v>42.40318845814829</v>
+        <v>42.34463278110177</v>
       </c>
       <c r="D2" t="n">
-        <v>38.42897173903754</v>
+        <v>53.81344159307785</v>
       </c>
       <c r="E2" t="n">
-        <v>41.581973407321</v>
+        <v>42.36485336705013</v>
       </c>
       <c r="F2" t="n">
-        <v>43.00892364678066</v>
+        <v>39.19642177180096</v>
       </c>
       <c r="G2" t="n">
-        <v>39.287269435033</v>
+        <v>45.48648281196142</v>
       </c>
       <c r="H2" t="n">
-        <v>48.3836768750091</v>
+        <v>52.03699095021992</v>
       </c>
       <c r="I2" t="n">
-        <v>32.51563453019705</v>
+        <v>42.72664144071113</v>
       </c>
       <c r="J2" t="n">
-        <v>48.80120895116702</v>
+        <v>48.59581065738591</v>
       </c>
       <c r="K2" t="n">
-        <v>45.5582388445243</v>
+        <v>46.02651922132481</v>
       </c>
       <c r="L2" t="n">
-        <v>45.05113597392727</v>
+        <v>44.58424506656207</v>
       </c>
     </row>
   </sheetData>
@@ -5826,37 +5826,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7043225420056842</v>
+        <v>159.0300293749897</v>
       </c>
       <c r="C2" t="n">
-        <v>38.82277320357824</v>
+        <v>41.31280124714651</v>
       </c>
       <c r="D2" t="n">
-        <v>35.3227133675224</v>
+        <v>36.14659092542262</v>
       </c>
       <c r="E2" t="n">
-        <v>34.99595905544398</v>
+        <v>42.34753581890011</v>
       </c>
       <c r="F2" t="n">
-        <v>42.62289935769812</v>
+        <v>49.29567155263253</v>
       </c>
       <c r="G2" t="n">
-        <v>37.45042346567558</v>
+        <v>39.49947012896655</v>
       </c>
       <c r="H2" t="n">
-        <v>42.0766055504904</v>
+        <v>43.00541815628471</v>
       </c>
       <c r="I2" t="n">
-        <v>36.0294397683412</v>
+        <v>46.95608629143095</v>
       </c>
       <c r="J2" t="n">
-        <v>31.96698698471366</v>
+        <v>34.81152436058287</v>
       </c>
       <c r="K2" t="n">
         <v>38.60546854285558</v>
       </c>
       <c r="L2" t="n">
-        <v>40.09070097999503</v>
+        <v>40.4521582230617</v>
       </c>
     </row>
   </sheetData>
@@ -5940,37 +5940,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6912223339895718</v>
+        <v>157.0919626660179</v>
       </c>
       <c r="C2" t="n">
-        <v>36.1139413692931</v>
+        <v>47.73265734167166</v>
       </c>
       <c r="D2" t="n">
-        <v>36.24312420957683</v>
+        <v>40.07184757569936</v>
       </c>
       <c r="E2" t="n">
-        <v>30.15281271055272</v>
+        <v>31.976615590194</v>
       </c>
       <c r="F2" t="n">
-        <v>35.84055592231252</v>
+        <v>42.31924848445949</v>
       </c>
       <c r="G2" t="n">
-        <v>36.61249484718294</v>
+        <v>37.04024421598007</v>
       </c>
       <c r="H2" t="n">
-        <v>53.67379734571858</v>
+        <v>60.25352914024463</v>
       </c>
       <c r="I2" t="n">
-        <v>41.88474015755338</v>
+        <v>46.46000725607838</v>
       </c>
       <c r="J2" t="n">
-        <v>47.82981115030486</v>
+        <v>51.50270213247768</v>
       </c>
       <c r="K2" t="n">
-        <v>40.73930999213975</v>
+        <v>48.07774610723385</v>
       </c>
       <c r="L2" t="n">
-        <v>38.9947803668584</v>
+        <v>44.01600517300673</v>
       </c>
     </row>
   </sheetData>
@@ -6054,37 +6054,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6943570839939639</v>
+        <v>156.7105847919593</v>
       </c>
       <c r="C2" t="n">
-        <v>48.27076373990897</v>
+        <v>52.92195288947391</v>
       </c>
       <c r="D2" t="n">
-        <v>53.2703368852049</v>
+        <v>53.03130790474333</v>
       </c>
       <c r="E2" t="n">
-        <v>47.16529252466633</v>
+        <v>47.03606593297118</v>
       </c>
       <c r="F2" t="n">
-        <v>39.82597990358001</v>
+        <v>41.67083203925993</v>
       </c>
       <c r="G2" t="n">
-        <v>46.21090554649456</v>
+        <v>46.01858154195121</v>
       </c>
       <c r="H2" t="n">
-        <v>43.15640159594155</v>
+        <v>56.0967505598022</v>
       </c>
       <c r="I2" t="n">
-        <v>54.99869054409848</v>
+        <v>52.39345907163957</v>
       </c>
       <c r="J2" t="n">
-        <v>37.65557022523262</v>
+        <v>45.09305807686439</v>
       </c>
       <c r="K2" t="n">
-        <v>40.22057805620729</v>
+        <v>43.35673914551324</v>
       </c>
       <c r="L2" t="n">
-        <v>37.13723882869608</v>
+        <v>41.12632722920956</v>
       </c>
     </row>
   </sheetData>
@@ -6168,37 +6168,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6510452089714818</v>
+        <v>147.3196788339992</v>
       </c>
       <c r="C2" t="n">
         <v>49.74205365006367</v>
       </c>
       <c r="D2" t="n">
-        <v>41.97557650606104</v>
+        <v>49.00238267999319</v>
       </c>
       <c r="E2" t="n">
-        <v>43.99619392966392</v>
+        <v>48.40888625093103</v>
       </c>
       <c r="F2" t="n">
         <v>38.55568052630458</v>
       </c>
       <c r="G2" t="n">
-        <v>41.2430942048604</v>
+        <v>45.98019743131452</v>
       </c>
       <c r="H2" t="n">
-        <v>39.98033854994674</v>
+        <v>41.56690590950648</v>
       </c>
       <c r="I2" t="n">
-        <v>33.47365382752751</v>
+        <v>38.35922724360001</v>
       </c>
       <c r="J2" t="n">
-        <v>42.31301728508722</v>
+        <v>42.70714214115564</v>
       </c>
       <c r="K2" t="n">
-        <v>37.6213678786184</v>
+        <v>37.55329415949174</v>
       </c>
       <c r="L2" t="n">
-        <v>39.97013824210564</v>
+        <v>44.77930346765061</v>
       </c>
     </row>
   </sheetData>
@@ -6282,37 +6282,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6902340829838067</v>
+        <v>156.4212254580343</v>
       </c>
       <c r="C2" t="n">
-        <v>32.98254565168146</v>
+        <v>37.8083996505012</v>
       </c>
       <c r="D2" t="n">
-        <v>40.28182773147263</v>
+        <v>46.17942743733445</v>
       </c>
       <c r="E2" t="n">
-        <v>31.39516101024411</v>
+        <v>36.48919265813847</v>
       </c>
       <c r="F2" t="n">
-        <v>40.02239118182934</v>
+        <v>43.8857527274367</v>
       </c>
       <c r="G2" t="n">
-        <v>30.9603996255237</v>
+        <v>29.94212632022764</v>
       </c>
       <c r="H2" t="n">
-        <v>45.95699605568232</v>
+        <v>49.77800192305625</v>
       </c>
       <c r="I2" t="n">
-        <v>38.14721061343781</v>
+        <v>41.24271044530561</v>
       </c>
       <c r="J2" t="n">
-        <v>42.78759924095779</v>
+        <v>42.62199408413018</v>
       </c>
       <c r="K2" t="n">
-        <v>42.84337681266752</v>
+        <v>45.2989279514743</v>
       </c>
       <c r="L2" t="n">
-        <v>47.32262989106156</v>
+        <v>47.29340851692817</v>
       </c>
     </row>
   </sheetData>
@@ -6396,37 +6396,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6627767080208287</v>
+        <v>150.1440514579881</v>
       </c>
       <c r="C2" t="n">
-        <v>39.75644702287984</v>
+        <v>37.93932893195843</v>
       </c>
       <c r="D2" t="n">
-        <v>41.63382245947945</v>
+        <v>45.42814854030308</v>
       </c>
       <c r="E2" t="n">
-        <v>35.83500486896882</v>
+        <v>35.73271258530085</v>
       </c>
       <c r="F2" t="n">
-        <v>40.44921997886823</v>
+        <v>54.71681075332513</v>
       </c>
       <c r="G2" t="n">
-        <v>30.46166889955701</v>
+        <v>30.58101999296436</v>
       </c>
       <c r="H2" t="n">
-        <v>47.97273301828424</v>
+        <v>62.01391736119704</v>
       </c>
       <c r="I2" t="n">
-        <v>35.72889586351747</v>
+        <v>35.5454108488796</v>
       </c>
       <c r="J2" t="n">
-        <v>36.74974976711251</v>
+        <v>37.16662526608019</v>
       </c>
       <c r="K2" t="n">
-        <v>38.63975526002081</v>
+        <v>45.22938566878194</v>
       </c>
       <c r="L2" t="n">
-        <v>54.31159830547914</v>
+        <v>53.75874120232885</v>
       </c>
     </row>
   </sheetData>
@@ -6510,37 +6510,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6371313750278205</v>
+        <v>146.4871718340437</v>
       </c>
       <c r="C2" t="n">
-        <v>45.01622392338524</v>
+        <v>45.76329604613203</v>
       </c>
       <c r="D2" t="n">
-        <v>56.90203642319787</v>
+        <v>57.66253914074893</v>
       </c>
       <c r="E2" t="n">
-        <v>46.66416978942468</v>
+        <v>47.14394663713669</v>
       </c>
       <c r="F2" t="n">
         <v>47.1633396043946</v>
       </c>
       <c r="G2" t="n">
-        <v>35.82684015253724</v>
+        <v>41.36017442521408</v>
       </c>
       <c r="H2" t="n">
-        <v>42.73575407531578</v>
+        <v>43.1140225445585</v>
       </c>
       <c r="I2" t="n">
-        <v>31.44210682695136</v>
+        <v>34.44089505280246</v>
       </c>
       <c r="J2" t="n">
-        <v>30.68141635046573</v>
+        <v>30.96279983753797</v>
       </c>
       <c r="K2" t="n">
-        <v>39.60264889848443</v>
+        <v>39.9840568051233</v>
       </c>
       <c r="L2" t="n">
-        <v>51.44044625076319</v>
+        <v>54.70139377769459</v>
       </c>
     </row>
   </sheetData>
@@ -6624,37 +6624,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6947256669518538</v>
+        <v>156.3998778329697</v>
       </c>
       <c r="C2" t="n">
-        <v>41.85982409237955</v>
+        <v>53.50425006405303</v>
       </c>
       <c r="D2" t="n">
         <v>44.04921811622263</v>
       </c>
       <c r="E2" t="n">
-        <v>42.69057881674752</v>
+        <v>42.63899347254788</v>
       </c>
       <c r="F2" t="n">
-        <v>35.3744906371056</v>
+        <v>44.40023854120739</v>
       </c>
       <c r="G2" t="n">
-        <v>31.59322591162984</v>
+        <v>39.96526435964577</v>
       </c>
       <c r="H2" t="n">
-        <v>38.86173601497406</v>
+        <v>40.72424412648649</v>
       </c>
       <c r="I2" t="n">
-        <v>18.30894358057951</v>
+        <v>18.51948892579748</v>
       </c>
       <c r="J2" t="n">
-        <v>39.74318700091469</v>
+        <v>39.74655220685159</v>
       </c>
       <c r="K2" t="n">
-        <v>42.38144430186753</v>
+        <v>53.0694049922088</v>
       </c>
       <c r="L2" t="n">
-        <v>44.54305486203778</v>
+        <v>44.67112153027075</v>
       </c>
     </row>
   </sheetData>
@@ -6738,34 +6738,34 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6533345420029946</v>
+        <v>147.0520283749793</v>
       </c>
       <c r="C2" t="n">
-        <v>46.45794513388842</v>
+        <v>50.06641846174421</v>
       </c>
       <c r="D2" t="n">
-        <v>48.65787366839543</v>
+        <v>53.57021581424679</v>
       </c>
       <c r="E2" t="n">
-        <v>40.57351424917817</v>
+        <v>44.05398145131072</v>
       </c>
       <c r="F2" t="n">
-        <v>41.03204221804343</v>
+        <v>45.02532833629573</v>
       </c>
       <c r="G2" t="n">
-        <v>27.26776905100474</v>
+        <v>33.06049437980644</v>
       </c>
       <c r="H2" t="n">
-        <v>27.68527388893607</v>
+        <v>31.95512085244698</v>
       </c>
       <c r="I2" t="n">
-        <v>50.83750450666026</v>
+        <v>47.93314725721931</v>
       </c>
       <c r="J2" t="n">
-        <v>42.33138741183349</v>
+        <v>48.03207841764119</v>
       </c>
       <c r="K2" t="n">
-        <v>39.46833091346325</v>
+        <v>39.14876477688263</v>
       </c>
       <c r="L2" t="n">
         <v>36.36194829399727</v>
@@ -6852,37 +6852,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6784592919866554</v>
+        <v>155.9505464159884</v>
       </c>
       <c r="C2" t="n">
-        <v>37.91460893482194</v>
+        <v>40.6320969725616</v>
       </c>
       <c r="D2" t="n">
-        <v>21.56402828069924</v>
+        <v>24.04366616221286</v>
       </c>
       <c r="E2" t="n">
-        <v>41.07874228617203</v>
+        <v>43.52976980141584</v>
       </c>
       <c r="F2" t="n">
-        <v>35.79928459801474</v>
+        <v>37.38263737343444</v>
       </c>
       <c r="G2" t="n">
-        <v>39.17327473042024</v>
+        <v>44.01991914053189</v>
       </c>
       <c r="H2" t="n">
-        <v>42.03138380561165</v>
+        <v>48.08474025824674</v>
       </c>
       <c r="I2" t="n">
-        <v>39.26672862674182</v>
+        <v>38.99087883536185</v>
       </c>
       <c r="J2" t="n">
-        <v>48.98932311257037</v>
+        <v>50.4507147872463</v>
       </c>
       <c r="K2" t="n">
-        <v>36.57734833308684</v>
+        <v>43.85105239844936</v>
       </c>
       <c r="L2" t="n">
-        <v>42.88146227655648</v>
+        <v>43.15610308638966</v>
       </c>
     </row>
   </sheetData>
@@ -6966,37 +6966,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7913587499642745</v>
+        <v>145.9271533749998</v>
       </c>
       <c r="C2" t="n">
-        <v>41.50118040776037</v>
+        <v>46.80953931430532</v>
       </c>
       <c r="D2" t="n">
-        <v>37.44548500262787</v>
+        <v>49.52898559385547</v>
       </c>
       <c r="E2" t="n">
-        <v>51.21560479929127</v>
+        <v>51.01841166954301</v>
       </c>
       <c r="F2" t="n">
-        <v>38.78971201959709</v>
+        <v>38.32676271378204</v>
       </c>
       <c r="G2" t="n">
-        <v>28.44160661171616</v>
+        <v>34.37311288420351</v>
       </c>
       <c r="H2" t="n">
-        <v>47.47397089694802</v>
+        <v>52.34001571203995</v>
       </c>
       <c r="I2" t="n">
-        <v>36.53692970573826</v>
+        <v>47.04614275458187</v>
       </c>
       <c r="J2" t="n">
-        <v>45.84876464739383</v>
+        <v>46.31409384680212</v>
       </c>
       <c r="K2" t="n">
-        <v>59.75151813038547</v>
+        <v>65.14104287662558</v>
       </c>
       <c r="L2" t="n">
-        <v>37.8385988960471</v>
+        <v>39.69067913615479</v>
       </c>
     </row>
   </sheetData>
@@ -7080,37 +7080,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6528279589838348</v>
+        <v>133.0683586660307</v>
       </c>
       <c r="C2" t="n">
-        <v>32.68980690791428</v>
+        <v>42.95251512624264</v>
       </c>
       <c r="D2" t="n">
-        <v>34.61152892698351</v>
+        <v>38.01075258695997</v>
       </c>
       <c r="E2" t="n">
-        <v>39.40898943856037</v>
+        <v>39.60952091192887</v>
       </c>
       <c r="F2" t="n">
-        <v>34.66486877159923</v>
+        <v>37.7391623870142</v>
       </c>
       <c r="G2" t="n">
-        <v>60.21052840687187</v>
+        <v>63.7750552002483</v>
       </c>
       <c r="H2" t="n">
-        <v>49.01489165025908</v>
+        <v>49.26911723831869</v>
       </c>
       <c r="I2" t="n">
-        <v>37.72124263545518</v>
+        <v>42.7427773330679</v>
       </c>
       <c r="J2" t="n">
-        <v>39.06704308892579</v>
+        <v>42.4326840927372</v>
       </c>
       <c r="K2" t="n">
-        <v>14.87353886780343</v>
+        <v>15.17230354899651</v>
       </c>
       <c r="L2" t="n">
-        <v>47.20851375784665</v>
+        <v>47.27127065492867</v>
       </c>
     </row>
   </sheetData>
@@ -7194,37 +7194,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6710315839736722</v>
+        <v>133.119712041982</v>
       </c>
       <c r="C2" t="n">
-        <v>39.45089430979953</v>
+        <v>40.45694113398862</v>
       </c>
       <c r="D2" t="n">
-        <v>39.83096222760857</v>
+        <v>47.92486394466922</v>
       </c>
       <c r="E2" t="n">
-        <v>35.97353269617837</v>
+        <v>36.24555181798642</v>
       </c>
       <c r="F2" t="n">
-        <v>30.38746090983773</v>
+        <v>30.4087121489545</v>
       </c>
       <c r="G2" t="n">
         <v>53.46087208404543</v>
       </c>
       <c r="H2" t="n">
-        <v>32.86919861320487</v>
+        <v>32.45741104705878</v>
       </c>
       <c r="I2" t="n">
-        <v>31.67288261489044</v>
+        <v>42.13953543776746</v>
       </c>
       <c r="J2" t="n">
-        <v>46.97115794373494</v>
+        <v>51.77681440410522</v>
       </c>
       <c r="K2" t="n">
-        <v>32.94000533790692</v>
+        <v>45.49412056345449</v>
       </c>
       <c r="L2" t="n">
-        <v>34.99565149380805</v>
+        <v>41.43546326235983</v>
       </c>
     </row>
   </sheetData>
@@ -7308,37 +7308,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6706727499840781</v>
+        <v>133.4925632920349</v>
       </c>
       <c r="C2" t="n">
-        <v>31.45041165443901</v>
+        <v>35.13696775814394</v>
       </c>
       <c r="D2" t="n">
-        <v>69.09593516366149</v>
+        <v>69.27178523035084</v>
       </c>
       <c r="E2" t="n">
-        <v>47.52155082971682</v>
+        <v>54.30855048544215</v>
       </c>
       <c r="F2" t="n">
-        <v>38.95706902401236</v>
+        <v>40.58851265449914</v>
       </c>
       <c r="G2" t="n">
-        <v>43.51298624989574</v>
+        <v>43.53724027614495</v>
       </c>
       <c r="H2" t="n">
-        <v>40.67435849323812</v>
+        <v>41.33730797209078</v>
       </c>
       <c r="I2" t="n">
-        <v>29.77688009609374</v>
+        <v>39.20999962300327</v>
       </c>
       <c r="J2" t="n">
-        <v>48.64649271205139</v>
+        <v>48.74963662854339</v>
       </c>
       <c r="K2" t="n">
-        <v>46.30062335528211</v>
+        <v>46.0212403272544</v>
       </c>
       <c r="L2" t="n">
-        <v>46.42275628792649</v>
+        <v>46.5510716149422</v>
       </c>
     </row>
   </sheetData>
@@ -7422,37 +7422,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6840127090108581</v>
+        <v>135.3965294159716</v>
       </c>
       <c r="C2" t="n">
-        <v>39.42073101759016</v>
+        <v>42.51645134618426</v>
       </c>
       <c r="D2" t="n">
-        <v>48.10273545726845</v>
+        <v>49.28113384256108</v>
       </c>
       <c r="E2" t="n">
-        <v>28.32632164943787</v>
+        <v>28.90566072869647</v>
       </c>
       <c r="F2" t="n">
         <v>46.88340152424848</v>
       </c>
       <c r="G2" t="n">
-        <v>48.39155525077568</v>
+        <v>47.96527276433446</v>
       </c>
       <c r="H2" t="n">
-        <v>40.50706699981107</v>
+        <v>46.30965485808247</v>
       </c>
       <c r="I2" t="n">
-        <v>40.31539369160505</v>
+        <v>40.32659001128162</v>
       </c>
       <c r="J2" t="n">
-        <v>38.87949885581156</v>
+        <v>45.72338179587829</v>
       </c>
       <c r="K2" t="n">
-        <v>54.78024346438085</v>
+        <v>55.25046232308891</v>
       </c>
       <c r="L2" t="n">
-        <v>47.95039088642623</v>
+        <v>45.81592944274411</v>
       </c>
     </row>
   </sheetData>
@@ -7536,37 +7536,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.666756916034501</v>
+        <v>133.0729502079776</v>
       </c>
       <c r="C2" t="n">
-        <v>43.3027913328885</v>
+        <v>46.38518938450446</v>
       </c>
       <c r="D2" t="n">
-        <v>53.66043831286741</v>
+        <v>56.5599278354812</v>
       </c>
       <c r="E2" t="n">
-        <v>49.05085073739018</v>
+        <v>54.42491112985761</v>
       </c>
       <c r="F2" t="n">
-        <v>42.78186006184799</v>
+        <v>47.77843862426789</v>
       </c>
       <c r="G2" t="n">
-        <v>38.46942641966157</v>
+        <v>39.13385677872923</v>
       </c>
       <c r="H2" t="n">
-        <v>40.25087892269009</v>
+        <v>40.68288108627495</v>
       </c>
       <c r="I2" t="n">
-        <v>45.43527726545909</v>
+        <v>48.15178131995056</v>
       </c>
       <c r="J2" t="n">
-        <v>34.5422181984199</v>
+        <v>40.16098038725692</v>
       </c>
       <c r="K2" t="n">
-        <v>47.87886006680775</v>
+        <v>47.63418287828749</v>
       </c>
       <c r="L2" t="n">
-        <v>37.64499902169509</v>
+        <v>42.37850678426716</v>
       </c>
     </row>
   </sheetData>
@@ -7650,37 +7650,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6926218750304542</v>
+        <v>136.2826885000104</v>
       </c>
       <c r="C2" t="n">
-        <v>39.53653340483583</v>
+        <v>58.11407540318756</v>
       </c>
       <c r="D2" t="n">
-        <v>37.66666149691</v>
+        <v>40.10466029429224</v>
       </c>
       <c r="E2" t="n">
-        <v>42.4841726754624</v>
+        <v>42.5146046652838</v>
       </c>
       <c r="F2" t="n">
-        <v>37.67807936049265</v>
+        <v>41.63794950516417</v>
       </c>
       <c r="G2" t="n">
-        <v>38.53282702019192</v>
+        <v>38.34299845112591</v>
       </c>
       <c r="H2" t="n">
-        <v>51.89938385280453</v>
+        <v>54.87648476003965</v>
       </c>
       <c r="I2" t="n">
-        <v>24.7156039998189</v>
+        <v>24.76724324733552</v>
       </c>
       <c r="J2" t="n">
         <v>46.86531926446545</v>
       </c>
       <c r="K2" t="n">
-        <v>54.01984335887837</v>
+        <v>55.52673122873016</v>
       </c>
       <c r="L2" t="n">
-        <v>43.73684076978272</v>
+        <v>60.79762271553587</v>
       </c>
     </row>
   </sheetData>
@@ -7764,37 +7764,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6784152499749325</v>
+        <v>134.5696824589977</v>
       </c>
       <c r="C2" t="n">
-        <v>38.17566638188902</v>
+        <v>48.21498324507517</v>
       </c>
       <c r="D2" t="n">
         <v>38.54243394496699</v>
       </c>
       <c r="E2" t="n">
-        <v>46.16928021587607</v>
+        <v>45.23227120689027</v>
       </c>
       <c r="F2" t="n">
-        <v>33.87957770366973</v>
+        <v>34.17647442613176</v>
       </c>
       <c r="G2" t="n">
-        <v>43.20812252882082</v>
+        <v>49.03190667459607</v>
       </c>
       <c r="H2" t="n">
-        <v>34.506379293542</v>
+        <v>42.03194817073645</v>
       </c>
       <c r="I2" t="n">
-        <v>38.04018045831292</v>
+        <v>44.54093867892774</v>
       </c>
       <c r="J2" t="n">
-        <v>31.69569949885099</v>
+        <v>41.01822006491268</v>
       </c>
       <c r="K2" t="n">
-        <v>36.64446501876885</v>
+        <v>48.55442506681827</v>
       </c>
       <c r="L2" t="n">
-        <v>41.90689904286119</v>
+        <v>46.56215882647053</v>
       </c>
     </row>
   </sheetData>
@@ -7878,37 +7878,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6649692920036614</v>
+        <v>133.0838016250054</v>
       </c>
       <c r="C2" t="n">
-        <v>35.4178271640214</v>
+        <v>35.73684381860846</v>
       </c>
       <c r="D2" t="n">
-        <v>27.22718733310859</v>
+        <v>27.61510048864348</v>
       </c>
       <c r="E2" t="n">
-        <v>46.44304432712423</v>
+        <v>46.12648018163114</v>
       </c>
       <c r="F2" t="n">
         <v>16.66663155055877</v>
       </c>
       <c r="G2" t="n">
-        <v>34.57459912361831</v>
+        <v>40.5544726380412</v>
       </c>
       <c r="H2" t="n">
-        <v>40.03219966830866</v>
+        <v>40.05745831401997</v>
       </c>
       <c r="I2" t="n">
-        <v>35.79373745862533</v>
+        <v>36.01527648414294</v>
       </c>
       <c r="J2" t="n">
-        <v>36.42821653443553</v>
+        <v>50.75401718828536</v>
       </c>
       <c r="K2" t="n">
-        <v>51.86606868177092</v>
+        <v>51.42966814164775</v>
       </c>
       <c r="L2" t="n">
-        <v>41.95667095164234</v>
+        <v>45.86227032911273</v>
       </c>
     </row>
   </sheetData>
@@ -7992,37 +7992,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6618940000189468</v>
+        <v>133.7050498750177</v>
       </c>
       <c r="C2" t="n">
-        <v>48.12951319190354</v>
+        <v>48.14340695064011</v>
       </c>
       <c r="D2" t="n">
         <v>53.88552489077368</v>
       </c>
       <c r="E2" t="n">
-        <v>41.45697474607929</v>
+        <v>42.77215936267494</v>
       </c>
       <c r="F2" t="n">
-        <v>40.56050679451636</v>
+        <v>40.38502275231005</v>
       </c>
       <c r="G2" t="n">
-        <v>29.29811768250764</v>
+        <v>37.60622075283534</v>
       </c>
       <c r="H2" t="n">
-        <v>42.58011735563414</v>
+        <v>47.69413038009893</v>
       </c>
       <c r="I2" t="n">
-        <v>31.90708255373931</v>
+        <v>32.14824835478919</v>
       </c>
       <c r="J2" t="n">
-        <v>35.79032634241664</v>
+        <v>36.76802430237373</v>
       </c>
       <c r="K2" t="n">
-        <v>34.46685187059048</v>
+        <v>50.60611894805105</v>
       </c>
       <c r="L2" t="n">
-        <v>46.60374238362404</v>
+        <v>46.53721571010899</v>
       </c>
     </row>
   </sheetData>
@@ -8106,37 +8106,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6356772500439547</v>
+        <v>129.2444874999928</v>
       </c>
       <c r="C2" t="n">
-        <v>46.66313464920998</v>
+        <v>50.22447085512069</v>
       </c>
       <c r="D2" t="n">
-        <v>48.27528437868538</v>
+        <v>57.08049602799319</v>
       </c>
       <c r="E2" t="n">
-        <v>33.77856384909045</v>
+        <v>34.26672462927151</v>
       </c>
       <c r="F2" t="n">
-        <v>37.85003658103615</v>
+        <v>37.31935032888887</v>
       </c>
       <c r="G2" t="n">
-        <v>47.1754222405841</v>
+        <v>47.73897201455118</v>
       </c>
       <c r="H2" t="n">
-        <v>45.33680623506415</v>
+        <v>45.04239896194132</v>
       </c>
       <c r="I2" t="n">
-        <v>43.61536560551261</v>
+        <v>43.8157551594165</v>
       </c>
       <c r="J2" t="n">
-        <v>43.27093604018997</v>
+        <v>53.38649821669785</v>
       </c>
       <c r="K2" t="n">
-        <v>35.83564489023661</v>
+        <v>36.25421808925585</v>
       </c>
       <c r="L2" t="n">
-        <v>34.12675008524005</v>
+        <v>38.73212837584211</v>
       </c>
     </row>
   </sheetData>
@@ -8220,37 +8220,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6388942080084234</v>
+        <v>134.8549677500268</v>
       </c>
       <c r="C2" t="n">
-        <v>31.43330775982816</v>
+        <v>40.12318572827191</v>
       </c>
       <c r="D2" t="n">
-        <v>35.76652380499289</v>
+        <v>40.3198092890062</v>
       </c>
       <c r="E2" t="n">
-        <v>46.20298148609901</v>
+        <v>45.79721896554783</v>
       </c>
       <c r="F2" t="n">
-        <v>49.14000954993851</v>
+        <v>48.87479932150092</v>
       </c>
       <c r="G2" t="n">
-        <v>39.21563758514624</v>
+        <v>38.45949739066109</v>
       </c>
       <c r="H2" t="n">
-        <v>39.46846523202936</v>
+        <v>47.4721758525384</v>
       </c>
       <c r="I2" t="n">
-        <v>45.59244435797503</v>
+        <v>46.21686247987229</v>
       </c>
       <c r="J2" t="n">
-        <v>34.48951884367386</v>
+        <v>35.88699449950038</v>
       </c>
       <c r="K2" t="n">
-        <v>34.87935038762144</v>
+        <v>34.98020661715508</v>
       </c>
       <c r="L2" t="n">
-        <v>44.29819131112264</v>
+        <v>43.82693051447113</v>
       </c>
     </row>
   </sheetData>
@@ -8334,37 +8334,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6859917499823496</v>
+        <v>139.1650577079854</v>
       </c>
       <c r="C2" t="n">
-        <v>44.37372936795713</v>
+        <v>44.92154063497759</v>
       </c>
       <c r="D2" t="n">
-        <v>42.12354790685691</v>
+        <v>41.57067138199992</v>
       </c>
       <c r="E2" t="n">
-        <v>38.40470243139736</v>
+        <v>47.07077350466061</v>
       </c>
       <c r="F2" t="n">
-        <v>36.15384618002118</v>
+        <v>43.10197434346021</v>
       </c>
       <c r="G2" t="n">
-        <v>35.00784291288304</v>
+        <v>35.80148519313158</v>
       </c>
       <c r="H2" t="n">
-        <v>30.12948855751518</v>
+        <v>35.80611106338311</v>
       </c>
       <c r="I2" t="n">
-        <v>32.16066742071132</v>
+        <v>31.93423169823491</v>
       </c>
       <c r="J2" t="n">
-        <v>34.59243794105069</v>
+        <v>34.19513262318378</v>
       </c>
       <c r="K2" t="n">
-        <v>39.86396234641442</v>
+        <v>50.18386414079207</v>
       </c>
       <c r="L2" t="n">
-        <v>32.86824354882828</v>
+        <v>32.98009336461242</v>
       </c>
     </row>
   </sheetData>
@@ -8448,37 +8448,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6769374590367079</v>
+        <v>138.8158990000375</v>
       </c>
       <c r="C2" t="n">
-        <v>62.51131528063725</v>
+        <v>63.0169702127937</v>
       </c>
       <c r="D2" t="n">
-        <v>41.82274108627852</v>
+        <v>47.53710559649647</v>
       </c>
       <c r="E2" t="n">
-        <v>39.37958155061315</v>
+        <v>38.92784381727181</v>
       </c>
       <c r="F2" t="n">
-        <v>64.61784891557551</v>
+        <v>65.33689148259879</v>
       </c>
       <c r="G2" t="n">
-        <v>31.86486219380767</v>
+        <v>37.58638851608048</v>
       </c>
       <c r="H2" t="n">
-        <v>45.42711405225523</v>
+        <v>44.10433265088818</v>
       </c>
       <c r="I2" t="n">
-        <v>40.97486358897509</v>
+        <v>43.12569493670293</v>
       </c>
       <c r="J2" t="n">
-        <v>36.58997347475766</v>
+        <v>42.84743873558887</v>
       </c>
       <c r="K2" t="n">
-        <v>34.41846948155369</v>
+        <v>47.91238271676944</v>
       </c>
       <c r="L2" t="n">
-        <v>42.14735519777027</v>
+        <v>51.69461999256639</v>
       </c>
     </row>
   </sheetData>
@@ -8562,37 +8562,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6649244159925729</v>
+        <v>134.4823769159848</v>
       </c>
       <c r="C2" t="n">
-        <v>63.60369962250034</v>
+        <v>63.01414560902267</v>
       </c>
       <c r="D2" t="n">
-        <v>48.22825851464558</v>
+        <v>52.95826604759674</v>
       </c>
       <c r="E2" t="n">
-        <v>47.88186119136418</v>
+        <v>58.17513430219601</v>
       </c>
       <c r="F2" t="n">
-        <v>48.24681688896861</v>
+        <v>47.24070320087061</v>
       </c>
       <c r="G2" t="n">
-        <v>41.61200298826575</v>
+        <v>50.8202501305495</v>
       </c>
       <c r="H2" t="n">
-        <v>41.12739164283407</v>
+        <v>40.81836201627114</v>
       </c>
       <c r="I2" t="n">
-        <v>40.84881945187296</v>
+        <v>48.98507997561933</v>
       </c>
       <c r="J2" t="n">
-        <v>34.86078776871282</v>
+        <v>34.89885886690413</v>
       </c>
       <c r="K2" t="n">
-        <v>44.49157906768249</v>
+        <v>51.90814842835498</v>
       </c>
       <c r="L2" t="n">
-        <v>50.70981705701411</v>
+        <v>50.5411327933823</v>
       </c>
     </row>
   </sheetData>
@@ -8676,37 +8676,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6655346669722348</v>
+        <v>146.2486261670128</v>
       </c>
       <c r="C2" t="n">
-        <v>58.92988502408817</v>
+        <v>58.4481328894812</v>
       </c>
       <c r="D2" t="n">
-        <v>48.44277942773002</v>
+        <v>48.74175001907174</v>
       </c>
       <c r="E2" t="n">
-        <v>35.58126838834441</v>
+        <v>36.34950029699723</v>
       </c>
       <c r="F2" t="n">
-        <v>31.44887168695905</v>
+        <v>31.64507065844025</v>
       </c>
       <c r="G2" t="n">
-        <v>44.13622465353065</v>
+        <v>45.81741966588103</v>
       </c>
       <c r="H2" t="n">
-        <v>31.89742457031442</v>
+        <v>38.75854033633696</v>
       </c>
       <c r="I2" t="n">
-        <v>41.50456705886042</v>
+        <v>43.05413010799072</v>
       </c>
       <c r="J2" t="n">
-        <v>55.76557356891057</v>
+        <v>57.70943046491222</v>
       </c>
       <c r="K2" t="n">
-        <v>55.77372382808036</v>
+        <v>51.34005872053692</v>
       </c>
       <c r="L2" t="n">
-        <v>48.13629336007916</v>
+        <v>47.89736713614855</v>
       </c>
     </row>
   </sheetData>
@@ -8790,37 +8790,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6736658749869093</v>
+        <v>194.8915444579907</v>
       </c>
       <c r="C2" t="n">
-        <v>44.07679277578714</v>
+        <v>44.35986385340818</v>
       </c>
       <c r="D2" t="n">
-        <v>33.03081649488477</v>
+        <v>42.95055189587862</v>
       </c>
       <c r="E2" t="n">
-        <v>33.39220733904304</v>
+        <v>40.31006796894926</v>
       </c>
       <c r="F2" t="n">
-        <v>33.31447063683147</v>
+        <v>44.01720544050235</v>
       </c>
       <c r="G2" t="n">
-        <v>43.76540424300766</v>
+        <v>45.15570636479706</v>
       </c>
       <c r="H2" t="n">
-        <v>45.28648065825737</v>
+        <v>51.20589902508542</v>
       </c>
       <c r="I2" t="n">
-        <v>31.93092476605001</v>
+        <v>39.16215359972514</v>
       </c>
       <c r="J2" t="n">
-        <v>38.09146950328119</v>
+        <v>38.17969316740795</v>
       </c>
       <c r="K2" t="n">
-        <v>31.23666833252891</v>
+        <v>31.38140053003002</v>
       </c>
       <c r="L2" t="n">
-        <v>27.76847537725181</v>
+        <v>32.5894140512809</v>
       </c>
     </row>
   </sheetData>
@@ -8904,37 +8904,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6472598750260659</v>
+        <v>192.0647389169899</v>
       </c>
       <c r="C2" t="n">
-        <v>41.60528197204412</v>
+        <v>42.51674439198514</v>
       </c>
       <c r="D2" t="n">
         <v>45.14254365801965</v>
       </c>
       <c r="E2" t="n">
-        <v>56.34198539452052</v>
+        <v>61.01494996820146</v>
       </c>
       <c r="F2" t="n">
-        <v>43.62074831522313</v>
+        <v>47.08752831539105</v>
       </c>
       <c r="G2" t="n">
-        <v>41.30966525983627</v>
+        <v>41.38786857521742</v>
       </c>
       <c r="H2" t="n">
-        <v>42.12233485436818</v>
+        <v>42.28418384030236</v>
       </c>
       <c r="I2" t="n">
         <v>41.950048854355</v>
       </c>
       <c r="J2" t="n">
-        <v>45.49534051520445</v>
+        <v>52.47124415340266</v>
       </c>
       <c r="K2" t="n">
-        <v>39.61858046476655</v>
+        <v>45.4103688009256</v>
       </c>
       <c r="L2" t="n">
-        <v>33.45550847109947</v>
+        <v>33.18765987022658</v>
       </c>
     </row>
   </sheetData>
@@ -9018,37 +9018,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.679747583984863</v>
+        <v>193.6448953750078</v>
       </c>
       <c r="C2" t="n">
-        <v>36.06917366640091</v>
+        <v>38.32264244303594</v>
       </c>
       <c r="D2" t="n">
-        <v>29.30508445968513</v>
+        <v>47.01169814670434</v>
       </c>
       <c r="E2" t="n">
-        <v>40.21349405732132</v>
+        <v>44.64180346674924</v>
       </c>
       <c r="F2" t="n">
-        <v>45.86851916494088</v>
+        <v>49.81272887667663</v>
       </c>
       <c r="G2" t="n">
-        <v>47.69621592742374</v>
+        <v>50.652829224349</v>
       </c>
       <c r="H2" t="n">
-        <v>32.73499481062986</v>
+        <v>32.99130023038777</v>
       </c>
       <c r="I2" t="n">
-        <v>47.32812464103996</v>
+        <v>55.15992311423106</v>
       </c>
       <c r="J2" t="n">
-        <v>58.16868895165841</v>
+        <v>58.13579514078634</v>
       </c>
       <c r="K2" t="n">
-        <v>31.61768595648689</v>
+        <v>31.81179446568506</v>
       </c>
       <c r="L2" t="n">
-        <v>49.54201150613791</v>
+        <v>48.15803865008291</v>
       </c>
     </row>
   </sheetData>
@@ -9132,37 +9132,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6884439580026083</v>
+        <v>197.6541770000476</v>
       </c>
       <c r="C2" t="n">
-        <v>39.87933538593099</v>
+        <v>46.36608461097055</v>
       </c>
       <c r="D2" t="n">
-        <v>40.1088527854829</v>
+        <v>44.83114404178225</v>
       </c>
       <c r="E2" t="n">
-        <v>43.26842681782892</v>
+        <v>43.55506813799862</v>
       </c>
       <c r="F2" t="n">
-        <v>37.91877962041531</v>
+        <v>42.68770894815449</v>
       </c>
       <c r="G2" t="n">
-        <v>40.56684265745658</v>
+        <v>40.76849263317541</v>
       </c>
       <c r="H2" t="n">
-        <v>49.01378734610211</v>
+        <v>49.05187910729725</v>
       </c>
       <c r="I2" t="n">
-        <v>30.07006735002648</v>
+        <v>30.17416044055586</v>
       </c>
       <c r="J2" t="n">
-        <v>40.16805150571169</v>
+        <v>40.00820769973527</v>
       </c>
       <c r="K2" t="n">
-        <v>37.50587568595673</v>
+        <v>43.37252307006996</v>
       </c>
       <c r="L2" t="n">
-        <v>36.73313466056961</v>
+        <v>41.26689537388856</v>
       </c>
     </row>
   </sheetData>
@@ -9246,37 +9246,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6996320419711992</v>
+        <v>161.4242966250167</v>
       </c>
       <c r="C2" t="n">
-        <v>35.71123496923395</v>
+        <v>38.38875554127545</v>
       </c>
       <c r="D2" t="n">
-        <v>40.27199491059212</v>
+        <v>44.06451998224492</v>
       </c>
       <c r="E2" t="n">
-        <v>35.42955544049335</v>
+        <v>39.5739247737193</v>
       </c>
       <c r="F2" t="n">
-        <v>34.4775842760882</v>
+        <v>34.61415534247632</v>
       </c>
       <c r="G2" t="n">
-        <v>40.60584746099536</v>
+        <v>41.67880186253884</v>
       </c>
       <c r="H2" t="n">
-        <v>33.97237644764073</v>
+        <v>34.18877132560115</v>
       </c>
       <c r="I2" t="n">
-        <v>37.03658037315371</v>
+        <v>38.22245287449653</v>
       </c>
       <c r="J2" t="n">
-        <v>49.44988956403913</v>
+        <v>49.92426873576094</v>
       </c>
       <c r="K2" t="n">
-        <v>45.12434850383497</v>
+        <v>50.07605561726743</v>
       </c>
       <c r="L2" t="n">
-        <v>39.23770347411967</v>
+        <v>39.63158433118367</v>
       </c>
     </row>
   </sheetData>
@@ -9360,37 +9360,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6650101250270382</v>
+        <v>139.0945412500296</v>
       </c>
       <c r="C2" t="n">
-        <v>38.63189411173707</v>
+        <v>38.69294270778277</v>
       </c>
       <c r="D2" t="n">
-        <v>47.66612111057959</v>
+        <v>50.26591548626849</v>
       </c>
       <c r="E2" t="n">
-        <v>40.62392840806446</v>
+        <v>48.22480659860879</v>
       </c>
       <c r="F2" t="n">
-        <v>49.86973220491738</v>
+        <v>58.48952271842767</v>
       </c>
       <c r="G2" t="n">
-        <v>36.71760798779393</v>
+        <v>39.71486662627461</v>
       </c>
       <c r="H2" t="n">
-        <v>38.65475763451362</v>
+        <v>42.11998404928741</v>
       </c>
       <c r="I2" t="n">
-        <v>28.89942558884365</v>
+        <v>36.20224064604702</v>
       </c>
       <c r="J2" t="n">
-        <v>30.23244745530285</v>
+        <v>34.302885960693</v>
       </c>
       <c r="K2" t="n">
-        <v>29.60345445769175</v>
+        <v>37.75645891918946</v>
       </c>
       <c r="L2" t="n">
-        <v>55.81464166077782</v>
+        <v>56.44879942190746</v>
       </c>
     </row>
   </sheetData>
@@ -9474,37 +9474,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.700636041990947</v>
+        <v>146.2931764160166</v>
       </c>
       <c r="C2" t="n">
-        <v>27.3321986112423</v>
+        <v>32.39280215929809</v>
       </c>
       <c r="D2" t="n">
-        <v>37.8521147893743</v>
+        <v>38.20159035212102</v>
       </c>
       <c r="E2" t="n">
-        <v>38.82222932409386</v>
+        <v>47.93840231508763</v>
       </c>
       <c r="F2" t="n">
-        <v>43.71334786116451</v>
+        <v>46.57127423546013</v>
       </c>
       <c r="G2" t="n">
-        <v>45.98354861646445</v>
+        <v>43.69617046964344</v>
       </c>
       <c r="H2" t="n">
-        <v>32.27513626400563</v>
+        <v>32.42703170720126</v>
       </c>
       <c r="I2" t="n">
-        <v>58.31134844686794</v>
+        <v>54.71814535998938</v>
       </c>
       <c r="J2" t="n">
-        <v>39.3643046004799</v>
+        <v>48.4771284549202</v>
       </c>
       <c r="K2" t="n">
-        <v>50.79754344006191</v>
+        <v>51.09841002000454</v>
       </c>
       <c r="L2" t="n">
-        <v>31.01139488352451</v>
+        <v>31.4380523370225</v>
       </c>
     </row>
   </sheetData>
@@ -9588,37 +9588,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6887591669801623</v>
+        <v>146.0152946250164</v>
       </c>
       <c r="C2" t="n">
-        <v>49.76749659557807</v>
+        <v>50.07196509564782</v>
       </c>
       <c r="D2" t="n">
-        <v>30.96270764997778</v>
+        <v>32.27983386762016</v>
       </c>
       <c r="E2" t="n">
-        <v>32.30426434951115</v>
+        <v>36.51532365532081</v>
       </c>
       <c r="F2" t="n">
-        <v>41.86247331729646</v>
+        <v>42.5177851452256</v>
       </c>
       <c r="G2" t="n">
-        <v>32.09005432558342</v>
+        <v>42.26790839943011</v>
       </c>
       <c r="H2" t="n">
-        <v>43.45972812017855</v>
+        <v>49.38904560096721</v>
       </c>
       <c r="I2" t="n">
-        <v>51.64571125001032</v>
+        <v>51.55653860412341</v>
       </c>
       <c r="J2" t="n">
-        <v>52.00980846128624</v>
+        <v>58.46048759015637</v>
       </c>
       <c r="K2" t="n">
-        <v>36.26906272760073</v>
+        <v>48.57947503789966</v>
       </c>
       <c r="L2" t="n">
-        <v>45.57144222205289</v>
+        <v>50.95710187106403</v>
       </c>
     </row>
   </sheetData>
@@ -9702,37 +9702,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6619415839668363</v>
+        <v>138.2734448330011</v>
       </c>
       <c r="C2" t="n">
-        <v>43.58691111198387</v>
+        <v>48.80546841718879</v>
       </c>
       <c r="D2" t="n">
-        <v>42.03919775223464</v>
+        <v>46.4165926360477</v>
       </c>
       <c r="E2" t="n">
-        <v>40.87997962610272</v>
+        <v>41.64516934803051</v>
       </c>
       <c r="F2" t="n">
-        <v>37.41864427451048</v>
+        <v>44.99326127619445</v>
       </c>
       <c r="G2" t="n">
-        <v>31.13889412231826</v>
+        <v>31.51493580812324</v>
       </c>
       <c r="H2" t="n">
-        <v>56.61518126595341</v>
+        <v>56.54424770216013</v>
       </c>
       <c r="I2" t="n">
-        <v>33.6035158727725</v>
+        <v>34.0287706286555</v>
       </c>
       <c r="J2" t="n">
-        <v>35.30602562742346</v>
+        <v>35.31420626909158</v>
       </c>
       <c r="K2" t="n">
-        <v>35.89756645683376</v>
+        <v>35.74016251487227</v>
       </c>
       <c r="L2" t="n">
-        <v>42.7932954329446</v>
+        <v>46.79287564760627</v>
       </c>
     </row>
   </sheetData>
@@ -9816,37 +9816,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.676571124990005</v>
+        <v>137.8228930000332</v>
       </c>
       <c r="C2" t="n">
-        <v>37.75590321645205</v>
+        <v>37.6713523988278</v>
       </c>
       <c r="D2" t="n">
-        <v>31.15500342902367</v>
+        <v>42.25819701465939</v>
       </c>
       <c r="E2" t="n">
-        <v>31.92429355681729</v>
+        <v>33.751140525922</v>
       </c>
       <c r="F2" t="n">
-        <v>36.68167770298787</v>
+        <v>36.68167770298788</v>
       </c>
       <c r="G2" t="n">
-        <v>33.6573327531632</v>
+        <v>33.65733275316321</v>
       </c>
       <c r="H2" t="n">
-        <v>56.42106263184249</v>
+        <v>55.55779159966423</v>
       </c>
       <c r="I2" t="n">
-        <v>36.16208212848072</v>
+        <v>40.80673844912565</v>
       </c>
       <c r="J2" t="n">
-        <v>43.26089262572744</v>
+        <v>45.93551458766398</v>
       </c>
       <c r="K2" t="n">
         <v>41.49690943112408</v>
       </c>
       <c r="L2" t="n">
-        <v>39.05993430161705</v>
+        <v>41.23360630658372</v>
       </c>
     </row>
   </sheetData>
@@ -9930,37 +9930,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6811635409831069</v>
+        <v>149.0107027920312</v>
       </c>
       <c r="C2" t="n">
-        <v>40.26956634003487</v>
+        <v>43.4813980132844</v>
       </c>
       <c r="D2" t="n">
-        <v>36.76648555161502</v>
+        <v>42.93740230103208</v>
       </c>
       <c r="E2" t="n">
-        <v>44.34456953167558</v>
+        <v>46.94488488907855</v>
       </c>
       <c r="F2" t="n">
-        <v>43.04892834605902</v>
+        <v>48.11639907310521</v>
       </c>
       <c r="G2" t="n">
-        <v>42.946798027783</v>
+        <v>50.23241093053407</v>
       </c>
       <c r="H2" t="n">
         <v>16.43979955007029</v>
       </c>
       <c r="I2" t="n">
-        <v>50.33363378693406</v>
+        <v>54.90836730752413</v>
       </c>
       <c r="J2" t="n">
-        <v>35.30933603746862</v>
+        <v>41.24819981841104</v>
       </c>
       <c r="K2" t="n">
-        <v>40.27060043320928</v>
+        <v>36.5446075288612</v>
       </c>
       <c r="L2" t="n">
-        <v>34.51735724357094</v>
+        <v>37.38002720400814</v>
       </c>
     </row>
   </sheetData>
@@ -10044,37 +10044,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7066372499684803</v>
+        <v>150.9004352919874</v>
       </c>
       <c r="C2" t="n">
-        <v>29.07938250863889</v>
+        <v>33.55582844464885</v>
       </c>
       <c r="D2" t="n">
-        <v>42.64007445749001</v>
+        <v>55.20341411427106</v>
       </c>
       <c r="E2" t="n">
-        <v>35.39880320852564</v>
+        <v>35.4546984304495</v>
       </c>
       <c r="F2" t="n">
-        <v>41.18109475946765</v>
+        <v>42.31426519099595</v>
       </c>
       <c r="G2" t="n">
-        <v>36.98735380110224</v>
+        <v>43.52972262231957</v>
       </c>
       <c r="H2" t="n">
-        <v>35.75869721224734</v>
+        <v>50.21335054638903</v>
       </c>
       <c r="I2" t="n">
-        <v>42.22987611853613</v>
+        <v>41.28877718574547</v>
       </c>
       <c r="J2" t="n">
-        <v>37.95407719611719</v>
+        <v>37.6957994664358</v>
       </c>
       <c r="K2" t="n">
-        <v>33.07725599810005</v>
+        <v>38.57890838340177</v>
       </c>
       <c r="L2" t="n">
-        <v>33.12759143515493</v>
+        <v>38.60803487533956</v>
       </c>
     </row>
   </sheetData>
@@ -10158,37 +10158,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6732668339973316</v>
+        <v>142.4104585419991</v>
       </c>
       <c r="C2" t="n">
-        <v>34.26230813763262</v>
+        <v>35.80742888857213</v>
       </c>
       <c r="D2" t="n">
-        <v>29.18715451318385</v>
+        <v>37.34591687636008</v>
       </c>
       <c r="E2" t="n">
-        <v>48.66653776837403</v>
+        <v>54.07696857635674</v>
       </c>
       <c r="F2" t="n">
-        <v>38.30290350845283</v>
+        <v>41.73838420167688</v>
       </c>
       <c r="G2" t="n">
-        <v>39.08297672455338</v>
+        <v>50.26008125206433</v>
       </c>
       <c r="H2" t="n">
-        <v>37.66602414097702</v>
+        <v>45.45571583846542</v>
       </c>
       <c r="I2" t="n">
-        <v>46.05965173758234</v>
+        <v>45.44076213616545</v>
       </c>
       <c r="J2" t="n">
-        <v>60.64174128512128</v>
+        <v>60.6913905357432</v>
       </c>
       <c r="K2" t="n">
-        <v>37.67277354985603</v>
+        <v>37.33240883400923</v>
       </c>
       <c r="L2" t="n">
-        <v>38.24501127098114</v>
+        <v>37.66517599060274</v>
       </c>
     </row>
   </sheetData>
@@ -10272,37 +10272,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6749094999977387</v>
+        <v>150.1232933340361</v>
       </c>
       <c r="C2" t="n">
-        <v>57.28160581838127</v>
+        <v>62.44036837690822</v>
       </c>
       <c r="D2" t="n">
-        <v>35.82143359510547</v>
+        <v>40.638426892779</v>
       </c>
       <c r="E2" t="n">
-        <v>32.61134873203449</v>
+        <v>36.63805268917324</v>
       </c>
       <c r="F2" t="n">
-        <v>43.16603068624315</v>
+        <v>42.86324245303646</v>
       </c>
       <c r="G2" t="n">
-        <v>46.91266418795599</v>
+        <v>50.9510514482073</v>
       </c>
       <c r="H2" t="n">
-        <v>38.0370807148505</v>
+        <v>38.13907743929099</v>
       </c>
       <c r="I2" t="n">
-        <v>47.46542449204992</v>
+        <v>47.05924263746926</v>
       </c>
       <c r="J2" t="n">
-        <v>60.44623668975104</v>
+        <v>60.95467936659826</v>
       </c>
       <c r="K2" t="n">
-        <v>36.53393254226607</v>
+        <v>43.90126575490139</v>
       </c>
       <c r="L2" t="n">
-        <v>35.44992814734424</v>
+        <v>35.07721502996184</v>
       </c>
     </row>
   </sheetData>
@@ -10386,37 +10386,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6437674579792656</v>
+        <v>137.2387613750179</v>
       </c>
       <c r="C2" t="n">
-        <v>50.54320888225768</v>
+        <v>51.37374331130157</v>
       </c>
       <c r="D2" t="n">
-        <v>37.36809249502561</v>
+        <v>42.75049131520696</v>
       </c>
       <c r="E2" t="n">
-        <v>36.33451516263286</v>
+        <v>38.66482456169885</v>
       </c>
       <c r="F2" t="n">
-        <v>34.22205625236179</v>
+        <v>38.08664448903908</v>
       </c>
       <c r="G2" t="n">
-        <v>48.3359961230548</v>
+        <v>48.80424450241306</v>
       </c>
       <c r="H2" t="n">
-        <v>56.11565526565423</v>
+        <v>56.62203111390365</v>
       </c>
       <c r="I2" t="n">
-        <v>51.94084449034825</v>
+        <v>52.08078680495753</v>
       </c>
       <c r="J2" t="n">
-        <v>47.79621823801343</v>
+        <v>47.85014664919083</v>
       </c>
       <c r="K2" t="n">
-        <v>37.34110816286586</v>
+        <v>43.63692468450174</v>
       </c>
       <c r="L2" t="n">
-        <v>37.77237479319804</v>
+        <v>45.36504749745419</v>
       </c>
     </row>
   </sheetData>
@@ -10500,37 +10500,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6590477080317214</v>
+        <v>138.0344235000084</v>
       </c>
       <c r="C2" t="n">
-        <v>39.36133380454995</v>
+        <v>45.11157633962297</v>
       </c>
       <c r="D2" t="n">
-        <v>35.22566459615228</v>
+        <v>39.00471388660292</v>
       </c>
       <c r="E2" t="n">
-        <v>38.72632547387291</v>
+        <v>46.20438693674316</v>
       </c>
       <c r="F2" t="n">
         <v>39.95725943187433</v>
       </c>
       <c r="G2" t="n">
-        <v>43.0546218765449</v>
+        <v>46.75782288487891</v>
       </c>
       <c r="H2" t="n">
-        <v>51.067497260627</v>
+        <v>51.18262848100847</v>
       </c>
       <c r="I2" t="n">
-        <v>39.04415112890467</v>
+        <v>39.23276893557523</v>
       </c>
       <c r="J2" t="n">
-        <v>38.60357530966766</v>
+        <v>59.57789202377921</v>
       </c>
       <c r="K2" t="n">
-        <v>35.55112476580614</v>
+        <v>35.58342507073583</v>
       </c>
       <c r="L2" t="n">
-        <v>43.95425184850541</v>
+        <v>46.04375500760577</v>
       </c>
     </row>
   </sheetData>
@@ -10614,37 +10614,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7149029999854974</v>
+        <v>149.7202669580001</v>
       </c>
       <c r="C2" t="n">
-        <v>38.45855087170636</v>
+        <v>53.44249671580831</v>
       </c>
       <c r="D2" t="n">
-        <v>43.93885498353</v>
+        <v>44.88175497876556</v>
       </c>
       <c r="E2" t="n">
         <v>40.3685124671552</v>
       </c>
       <c r="F2" t="n">
-        <v>29.75924340264368</v>
+        <v>34.93675223219806</v>
       </c>
       <c r="G2" t="n">
-        <v>46.30340034990783</v>
+        <v>56.08665865598372</v>
       </c>
       <c r="H2" t="n">
-        <v>41.93435412390945</v>
+        <v>47.41390277465948</v>
       </c>
       <c r="I2" t="n">
-        <v>47.29203499512778</v>
+        <v>46.91271726175685</v>
       </c>
       <c r="J2" t="n">
-        <v>43.82911627821695</v>
+        <v>47.39282056733036</v>
       </c>
       <c r="K2" t="n">
-        <v>48.71843296945619</v>
+        <v>48.92794093700988</v>
       </c>
       <c r="L2" t="n">
-        <v>36.89930203684494</v>
+        <v>41.59354279853959</v>
       </c>
     </row>
   </sheetData>
@@ -10728,37 +10728,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7420707080163993</v>
+        <v>144.0142094999901</v>
       </c>
       <c r="C2" t="n">
-        <v>32.0534457563831</v>
+        <v>35.80984558165363</v>
       </c>
       <c r="D2" t="n">
-        <v>29.754905615652</v>
+        <v>29.92471993572786</v>
       </c>
       <c r="E2" t="n">
-        <v>46.16446828135841</v>
+        <v>53.68804694918752</v>
       </c>
       <c r="F2" t="n">
-        <v>46.67093224543128</v>
+        <v>50.06389511174995</v>
       </c>
       <c r="G2" t="n">
-        <v>44.20363693347656</v>
+        <v>52.15882722026409</v>
       </c>
       <c r="H2" t="n">
-        <v>44.61639883885658</v>
+        <v>51.45359409074842</v>
       </c>
       <c r="I2" t="n">
-        <v>44.82393019508518</v>
+        <v>47.18840338426051</v>
       </c>
       <c r="J2" t="n">
-        <v>45.82778968779756</v>
+        <v>45.92188764350287</v>
       </c>
       <c r="K2" t="n">
-        <v>26.7636883214236</v>
+        <v>31.05371978838627</v>
       </c>
       <c r="L2" t="n">
-        <v>42.57808865993258</v>
+        <v>47.21086729561668</v>
       </c>
     </row>
   </sheetData>
@@ -10842,37 +10842,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6343577500083484</v>
+        <v>134.5106049170136</v>
       </c>
       <c r="C2" t="n">
-        <v>48.05583947827066</v>
+        <v>51.12259761073076</v>
       </c>
       <c r="D2" t="n">
-        <v>32.32958681964016</v>
+        <v>32.06236897542365</v>
       </c>
       <c r="E2" t="n">
-        <v>38.27273420712822</v>
+        <v>42.29204865448605</v>
       </c>
       <c r="F2" t="n">
-        <v>49.57929048193881</v>
+        <v>50.21561140611165</v>
       </c>
       <c r="G2" t="n">
-        <v>44.86840642984019</v>
+        <v>45.25980846990991</v>
       </c>
       <c r="H2" t="n">
-        <v>40.96686541899659</v>
+        <v>46.09001824993612</v>
       </c>
       <c r="I2" t="n">
-        <v>59.1393989011391</v>
+        <v>59.79659774044185</v>
       </c>
       <c r="J2" t="n">
-        <v>43.82636323212309</v>
+        <v>43.44724379626098</v>
       </c>
       <c r="K2" t="n">
         <v>49.94674490807952</v>
       </c>
       <c r="L2" t="n">
-        <v>29.85213821447872</v>
+        <v>41.227116905458</v>
       </c>
     </row>
   </sheetData>
@@ -10956,37 +10956,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6790455000009388</v>
+        <v>141.6398607919691</v>
       </c>
       <c r="C2" t="n">
-        <v>22.80914392813674</v>
+        <v>28.69463720426232</v>
       </c>
       <c r="D2" t="n">
-        <v>33.82642708945543</v>
+        <v>44.76557453549095</v>
       </c>
       <c r="E2" t="n">
-        <v>38.37360010421734</v>
+        <v>40.20145384701793</v>
       </c>
       <c r="F2" t="n">
-        <v>66.37376128761922</v>
+        <v>66.072787806999</v>
       </c>
       <c r="G2" t="n">
-        <v>29.8435754272591</v>
+        <v>34.60850103996405</v>
       </c>
       <c r="H2" t="n">
         <v>39.90584642561835</v>
       </c>
       <c r="I2" t="n">
-        <v>49.69277376776752</v>
+        <v>57.5125554622282</v>
       </c>
       <c r="J2" t="n">
-        <v>37.50824873860172</v>
+        <v>40.20810427019327</v>
       </c>
       <c r="K2" t="n">
-        <v>45.75675546864126</v>
+        <v>46.29377778315042</v>
       </c>
       <c r="L2" t="n">
-        <v>41.58050868769374</v>
+        <v>42.10902787344789</v>
       </c>
     </row>
   </sheetData>
@@ -11070,37 +11070,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6677437499747612</v>
+        <v>137.3391549999942</v>
       </c>
       <c r="C2" t="n">
-        <v>47.05910053133646</v>
+        <v>52.42403165841395</v>
       </c>
       <c r="D2" t="n">
-        <v>38.39313699082916</v>
+        <v>38.44985753787494</v>
       </c>
       <c r="E2" t="n">
-        <v>33.05297460786935</v>
+        <v>39.23405906105134</v>
       </c>
       <c r="F2" t="n">
         <v>29.62053461280191</v>
       </c>
       <c r="G2" t="n">
-        <v>48.14830986551969</v>
+        <v>48.30988731365819</v>
       </c>
       <c r="H2" t="n">
-        <v>48.89785870973792</v>
+        <v>49.0480015164743</v>
       </c>
       <c r="I2" t="n">
-        <v>43.92829540041848</v>
+        <v>44.42878768351531</v>
       </c>
       <c r="J2" t="n">
-        <v>38.48843039970777</v>
+        <v>38.66786970395171</v>
       </c>
       <c r="K2" t="n">
-        <v>42.48909530728874</v>
+        <v>42.53745992899991</v>
       </c>
       <c r="L2" t="n">
-        <v>32.47068501727916</v>
+        <v>40.90494102190377</v>
       </c>
     </row>
   </sheetData>
@@ -11184,37 +11184,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6469265419873409</v>
+        <v>135.7288320420193</v>
       </c>
       <c r="C2" t="n">
-        <v>20.99180833568746</v>
+        <v>22.61812957637882</v>
       </c>
       <c r="D2" t="n">
-        <v>27.13787292435108</v>
+        <v>27.25395637382929</v>
       </c>
       <c r="E2" t="n">
-        <v>52.22760208512888</v>
+        <v>56.42106521836833</v>
       </c>
       <c r="F2" t="n">
-        <v>47.25548617871966</v>
+        <v>46.90086457961215</v>
       </c>
       <c r="G2" t="n">
-        <v>45.14143252935824</v>
+        <v>54.08906893003331</v>
       </c>
       <c r="H2" t="n">
-        <v>37.40375899403196</v>
+        <v>52.10895653637578</v>
       </c>
       <c r="I2" t="n">
-        <v>40.28691059103154</v>
+        <v>42.96124403339879</v>
       </c>
       <c r="J2" t="n">
-        <v>32.55653890084961</v>
+        <v>33.18911978738564</v>
       </c>
       <c r="K2" t="n">
-        <v>35.10834403952596</v>
+        <v>35.21258049849137</v>
       </c>
       <c r="L2" t="n">
-        <v>59.97034011272522</v>
+        <v>62.81052260709096</v>
       </c>
     </row>
   </sheetData>
@@ -11298,37 +11298,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6327356660040095</v>
+        <v>132.0166811250383</v>
       </c>
       <c r="C2" t="n">
-        <v>32.15773590774006</v>
+        <v>32.93630806145946</v>
       </c>
       <c r="D2" t="n">
-        <v>42.88264664806587</v>
+        <v>46.65707222035712</v>
       </c>
       <c r="E2" t="n">
-        <v>41.49316480743701</v>
+        <v>40.71052096993584</v>
       </c>
       <c r="F2" t="n">
-        <v>43.39062005388531</v>
+        <v>48.36367200731293</v>
       </c>
       <c r="G2" t="n">
-        <v>36.94470546067058</v>
+        <v>40.23548746959933</v>
       </c>
       <c r="H2" t="n">
-        <v>42.31556574018398</v>
+        <v>41.51987692327867</v>
       </c>
       <c r="I2" t="n">
-        <v>41.21576466940095</v>
+        <v>41.37729603319892</v>
       </c>
       <c r="J2" t="n">
-        <v>43.35425694470592</v>
+        <v>43.64409252533873</v>
       </c>
       <c r="K2" t="n">
-        <v>32.90252229837401</v>
+        <v>32.78859092060482</v>
       </c>
       <c r="L2" t="n">
-        <v>35.07398839502144</v>
+        <v>47.89689593862166</v>
       </c>
     </row>
   </sheetData>
@@ -11412,37 +11412,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6412740839878097</v>
+        <v>133.6890992919798</v>
       </c>
       <c r="C2" t="n">
-        <v>42.208807886976</v>
+        <v>46.89868130900764</v>
       </c>
       <c r="D2" t="n">
-        <v>30.90658649492695</v>
+        <v>33.916498125697</v>
       </c>
       <c r="E2" t="n">
-        <v>56.63052774131589</v>
+        <v>57.08812009384478</v>
       </c>
       <c r="F2" t="n">
         <v>42.4270690785375</v>
       </c>
       <c r="G2" t="n">
-        <v>55.59166470422981</v>
+        <v>57.56076388804754</v>
       </c>
       <c r="H2" t="n">
-        <v>30.16747272822337</v>
+        <v>35.6653185208955</v>
       </c>
       <c r="I2" t="n">
-        <v>27.34452122443817</v>
+        <v>30.00322381217483</v>
       </c>
       <c r="J2" t="n">
-        <v>46.94332233961115</v>
+        <v>53.10448798621228</v>
       </c>
       <c r="K2" t="n">
-        <v>36.48830141482818</v>
+        <v>36.2093798546773</v>
       </c>
       <c r="L2" t="n">
-        <v>42.90260468297077</v>
+        <v>46.94524213833123</v>
       </c>
     </row>
   </sheetData>
@@ -11526,37 +11526,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7109319999581203</v>
+        <v>146.9515762500232</v>
       </c>
       <c r="C2" t="n">
-        <v>51.9969078801936</v>
+        <v>55.37827613692065</v>
       </c>
       <c r="D2" t="n">
-        <v>48.80624934324866</v>
+        <v>53.63744305479124</v>
       </c>
       <c r="E2" t="n">
-        <v>46.83311039802502</v>
+        <v>53.27592284454591</v>
       </c>
       <c r="F2" t="n">
-        <v>34.40113573385678</v>
+        <v>43.63454217060399</v>
       </c>
       <c r="G2" t="n">
-        <v>44.53229704712641</v>
+        <v>47.64082413384211</v>
       </c>
       <c r="H2" t="n">
-        <v>35.64673439332155</v>
+        <v>37.31830948853869</v>
       </c>
       <c r="I2" t="n">
-        <v>36.08236208811939</v>
+        <v>36.43458356539843</v>
       </c>
       <c r="J2" t="n">
-        <v>42.00924991185774</v>
+        <v>48.79694289790948</v>
       </c>
       <c r="K2" t="n">
         <v>65.50067318202021</v>
       </c>
       <c r="L2" t="n">
-        <v>47.41964448036108</v>
+        <v>56.12190642714988</v>
       </c>
     </row>
   </sheetData>
@@ -11640,37 +11640,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7116936250240542</v>
+        <v>147.5082176660071</v>
       </c>
       <c r="C2" t="n">
-        <v>39.00269949026888</v>
+        <v>51.71548634210162</v>
       </c>
       <c r="D2" t="n">
-        <v>48.09620760860119</v>
+        <v>48.20771414888267</v>
       </c>
       <c r="E2" t="n">
         <v>35.6236285492549</v>
       </c>
       <c r="F2" t="n">
-        <v>33.10608431211022</v>
+        <v>40.96526474428418</v>
       </c>
       <c r="G2" t="n">
-        <v>55.14337501464468</v>
+        <v>55.62946512638673</v>
       </c>
       <c r="H2" t="n">
-        <v>24.8407129129849</v>
+        <v>25.14404016263266</v>
       </c>
       <c r="I2" t="n">
-        <v>45.41395480016617</v>
+        <v>50.62431826899878</v>
       </c>
       <c r="J2" t="n">
-        <v>56.81504955507161</v>
+        <v>62.01797842335339</v>
       </c>
       <c r="K2" t="n">
-        <v>50.8793615197066</v>
+        <v>50.55335984096846</v>
       </c>
       <c r="L2" t="n">
-        <v>38.34279019148406</v>
+        <v>39.92788369179346</v>
       </c>
     </row>
   </sheetData>
@@ -11754,37 +11754,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6688030000077561</v>
+        <v>138.1042588330456</v>
       </c>
       <c r="C2" t="n">
-        <v>34.35562267794691</v>
+        <v>38.06744664185384</v>
       </c>
       <c r="D2" t="n">
-        <v>55.47685485504267</v>
+        <v>54.87922323297204</v>
       </c>
       <c r="E2" t="n">
-        <v>43.33231745268643</v>
+        <v>43.52955216853627</v>
       </c>
       <c r="F2" t="n">
-        <v>44.62572617955334</v>
+        <v>51.66252248599366</v>
       </c>
       <c r="G2" t="n">
-        <v>37.54856470237311</v>
+        <v>40.78627657887483</v>
       </c>
       <c r="H2" t="n">
-        <v>44.63251384914961</v>
+        <v>45.71527066871348</v>
       </c>
       <c r="I2" t="n">
-        <v>51.61852515730368</v>
+        <v>51.64432076511851</v>
       </c>
       <c r="J2" t="n">
         <v>38.69220311619873</v>
       </c>
       <c r="K2" t="n">
-        <v>37.13437161193936</v>
+        <v>37.06542984936836</v>
       </c>
       <c r="L2" t="n">
-        <v>48.33363348658519</v>
+        <v>41.94680677355695</v>
       </c>
     </row>
   </sheetData>
@@ -11868,37 +11868,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.666316042013932</v>
+        <v>135.8356473330059</v>
       </c>
       <c r="C2" t="n">
-        <v>51.11816656876152</v>
+        <v>54.01357312220054</v>
       </c>
       <c r="D2" t="n">
-        <v>42.44621920514684</v>
+        <v>42.31953838084871</v>
       </c>
       <c r="E2" t="n">
-        <v>34.78575284585926</v>
+        <v>49.5134342573449</v>
       </c>
       <c r="F2" t="n">
-        <v>31.59107291779814</v>
+        <v>31.61896559722033</v>
       </c>
       <c r="G2" t="n">
-        <v>32.32463925384028</v>
+        <v>32.76971650638785</v>
       </c>
       <c r="H2" t="n">
-        <v>34.97224789593143</v>
+        <v>36.56039100986463</v>
       </c>
       <c r="I2" t="n">
-        <v>47.9181303308177</v>
+        <v>49.64843115529821</v>
       </c>
       <c r="J2" t="n">
-        <v>40.14999922459543</v>
+        <v>40.61410951943834</v>
       </c>
       <c r="K2" t="n">
-        <v>42.73742781307568</v>
+        <v>44.7482538369791</v>
       </c>
       <c r="L2" t="n">
-        <v>37.05680057667082</v>
+        <v>45.5449531265141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>